<commit_message>
MMS does no longer check further paths if a non empty value already has been found
</commit_message>
<xml_diff>
--- a/stationsinformation.xlsx
+++ b/stationsinformation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="265">
   <si>
     <t>Device</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t>MZ Automation</t>
-  </si>
-  <si>
-    <t>1.3.0</t>
   </si>
   <si>
     <t>127.0.0.2</t>
@@ -1179,9 +1176,6 @@
       <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" t="s">
         <v>9</v>
       </c>
@@ -1191,7 +1185,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
         <v>9</v>
@@ -1202,7 +1196,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
         <v>9</v>
@@ -1213,7 +1207,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
         <v>9</v>
@@ -1224,7 +1218,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6" t="s">
         <v>9</v>
@@ -1235,7 +1229,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G7" t="s">
         <v>9</v>
@@ -1246,7 +1240,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
         <v>9</v>
@@ -1257,7 +1251,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" t="s">
         <v>9</v>
@@ -1268,7 +1262,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G10" t="s">
         <v>9</v>
@@ -1279,7 +1273,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G11" t="s">
         <v>9</v>
@@ -1290,7 +1284,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G12" t="s">
         <v>9</v>
@@ -1301,7 +1295,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" t="s">
         <v>9</v>
@@ -1312,7 +1306,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
         <v>9</v>
@@ -1323,7 +1317,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G15" t="s">
         <v>9</v>
@@ -1334,7 +1328,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G16" t="s">
         <v>9</v>
@@ -1345,7 +1339,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G17" t="s">
         <v>9</v>
@@ -1356,7 +1350,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G18" t="s">
         <v>9</v>
@@ -1367,7 +1361,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G19" t="s">
         <v>9</v>
@@ -1378,7 +1372,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G20" t="s">
         <v>9</v>
@@ -1389,7 +1383,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G21" t="s">
         <v>9</v>
@@ -1400,7 +1394,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G22" t="s">
         <v>9</v>
@@ -1411,7 +1405,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G23" t="s">
         <v>9</v>
@@ -1422,7 +1416,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G24" t="s">
         <v>9</v>
@@ -1433,7 +1427,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G25" t="s">
         <v>9</v>
@@ -1444,7 +1438,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G26" t="s">
         <v>9</v>
@@ -1455,7 +1449,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G27" t="s">
         <v>9</v>
@@ -1466,7 +1460,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G28" t="s">
         <v>9</v>
@@ -1477,7 +1471,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G29" t="s">
         <v>9</v>
@@ -1488,7 +1482,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G30" t="s">
         <v>9</v>
@@ -1499,7 +1493,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G31" t="s">
         <v>9</v>
@@ -1510,7 +1504,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G32" t="s">
         <v>9</v>
@@ -1521,7 +1515,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G33" t="s">
         <v>9</v>
@@ -1532,7 +1526,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G34" t="s">
         <v>9</v>
@@ -1543,7 +1537,7 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G35" t="s">
         <v>9</v>
@@ -1554,7 +1548,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G36" t="s">
         <v>9</v>
@@ -1565,7 +1559,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G37" t="s">
         <v>9</v>
@@ -1576,7 +1570,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G38" t="s">
         <v>9</v>
@@ -1587,7 +1581,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G39" t="s">
         <v>9</v>
@@ -1598,7 +1592,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G40" t="s">
         <v>9</v>
@@ -1609,7 +1603,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G41" t="s">
         <v>9</v>
@@ -1620,7 +1614,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G42" t="s">
         <v>9</v>
@@ -1631,7 +1625,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G43" t="s">
         <v>9</v>
@@ -1642,7 +1636,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G44" t="s">
         <v>9</v>
@@ -1653,7 +1647,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G45" t="s">
         <v>9</v>
@@ -1664,7 +1658,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G46" t="s">
         <v>9</v>
@@ -1675,7 +1669,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G47" t="s">
         <v>9</v>
@@ -1686,7 +1680,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G48" t="s">
         <v>9</v>
@@ -1697,7 +1691,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G49" t="s">
         <v>9</v>
@@ -1708,7 +1702,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G50" t="s">
         <v>9</v>
@@ -1719,7 +1713,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G51" t="s">
         <v>9</v>
@@ -1730,7 +1724,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G52" t="s">
         <v>9</v>
@@ -1741,7 +1735,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G53" t="s">
         <v>9</v>
@@ -1752,7 +1746,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G54" t="s">
         <v>9</v>
@@ -1763,7 +1757,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G55" t="s">
         <v>9</v>
@@ -1774,7 +1768,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G56" t="s">
         <v>9</v>
@@ -1785,7 +1779,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G57" t="s">
         <v>9</v>
@@ -1796,7 +1790,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G58" t="s">
         <v>9</v>
@@ -1807,7 +1801,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G59" t="s">
         <v>9</v>
@@ -1818,7 +1812,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G60" t="s">
         <v>9</v>
@@ -1829,7 +1823,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G61" t="s">
         <v>9</v>
@@ -1840,7 +1834,7 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G62" t="s">
         <v>9</v>
@@ -1851,7 +1845,7 @@
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G63" t="s">
         <v>9</v>
@@ -1862,7 +1856,7 @@
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G64" t="s">
         <v>9</v>
@@ -1873,7 +1867,7 @@
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G65" t="s">
         <v>9</v>
@@ -1884,7 +1878,7 @@
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G66" t="s">
         <v>9</v>
@@ -1895,7 +1889,7 @@
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G67" t="s">
         <v>9</v>
@@ -1906,7 +1900,7 @@
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G68" t="s">
         <v>9</v>
@@ -1917,7 +1911,7 @@
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G69" t="s">
         <v>9</v>
@@ -1928,7 +1922,7 @@
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G70" t="s">
         <v>9</v>
@@ -1939,7 +1933,7 @@
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G71" t="s">
         <v>9</v>
@@ -1950,7 +1944,7 @@
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G72" t="s">
         <v>9</v>
@@ -1961,7 +1955,7 @@
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G73" t="s">
         <v>9</v>
@@ -1972,7 +1966,7 @@
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G74" t="s">
         <v>9</v>
@@ -1983,7 +1977,7 @@
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G75" t="s">
         <v>9</v>
@@ -1994,7 +1988,7 @@
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G76" t="s">
         <v>9</v>
@@ -2005,7 +1999,7 @@
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G77" t="s">
         <v>9</v>
@@ -2016,7 +2010,7 @@
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G78" t="s">
         <v>9</v>
@@ -2027,7 +2021,7 @@
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G79" t="s">
         <v>9</v>
@@ -2038,7 +2032,7 @@
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G80" t="s">
         <v>9</v>
@@ -2049,7 +2043,7 @@
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G81" t="s">
         <v>9</v>
@@ -2060,7 +2054,7 @@
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G82" t="s">
         <v>9</v>
@@ -2071,7 +2065,7 @@
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G83" t="s">
         <v>9</v>
@@ -2082,7 +2076,7 @@
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G84" t="s">
         <v>9</v>
@@ -2093,7 +2087,7 @@
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G85" t="s">
         <v>9</v>
@@ -2104,7 +2098,7 @@
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G86" t="s">
         <v>9</v>
@@ -2115,7 +2109,7 @@
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G87" t="s">
         <v>9</v>
@@ -2126,7 +2120,7 @@
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G88" t="s">
         <v>9</v>
@@ -2137,7 +2131,7 @@
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G89" t="s">
         <v>9</v>
@@ -2148,7 +2142,7 @@
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G90" t="s">
         <v>9</v>
@@ -2159,7 +2153,7 @@
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G91" t="s">
         <v>9</v>
@@ -2170,7 +2164,7 @@
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G92" t="s">
         <v>9</v>
@@ -2181,7 +2175,7 @@
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G93" t="s">
         <v>9</v>
@@ -2192,7 +2186,7 @@
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G94" t="s">
         <v>9</v>
@@ -2203,7 +2197,7 @@
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G95" t="s">
         <v>9</v>
@@ -2214,7 +2208,7 @@
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G96" t="s">
         <v>9</v>
@@ -2225,7 +2219,7 @@
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G97" t="s">
         <v>9</v>
@@ -2236,7 +2230,7 @@
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G98" t="s">
         <v>9</v>
@@ -2247,7 +2241,7 @@
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G99" t="s">
         <v>9</v>
@@ -2258,7 +2252,7 @@
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G100" t="s">
         <v>9</v>
@@ -2269,7 +2263,7 @@
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G101" t="s">
         <v>9</v>
@@ -2280,7 +2274,7 @@
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G102" t="s">
         <v>9</v>
@@ -2291,7 +2285,7 @@
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G103" t="s">
         <v>9</v>
@@ -2302,7 +2296,7 @@
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G104" t="s">
         <v>9</v>
@@ -2313,7 +2307,7 @@
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G105" t="s">
         <v>9</v>
@@ -2324,7 +2318,7 @@
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G106" t="s">
         <v>9</v>
@@ -2335,7 +2329,7 @@
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G107" t="s">
         <v>9</v>
@@ -2346,7 +2340,7 @@
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G108" t="s">
         <v>9</v>
@@ -2357,7 +2351,7 @@
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G109" t="s">
         <v>9</v>
@@ -2368,7 +2362,7 @@
     </row>
     <row r="110" spans="1:8">
       <c r="A110" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G110" t="s">
         <v>9</v>
@@ -2379,7 +2373,7 @@
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G111" t="s">
         <v>9</v>
@@ -2390,7 +2384,7 @@
     </row>
     <row r="112" spans="1:8">
       <c r="A112" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G112" t="s">
         <v>9</v>
@@ -2401,7 +2395,7 @@
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G113" t="s">
         <v>9</v>
@@ -2412,7 +2406,7 @@
     </row>
     <row r="114" spans="1:8">
       <c r="A114" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G114" t="s">
         <v>9</v>
@@ -2423,7 +2417,7 @@
     </row>
     <row r="115" spans="1:8">
       <c r="A115" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G115" t="s">
         <v>9</v>
@@ -2434,7 +2428,7 @@
     </row>
     <row r="116" spans="1:8">
       <c r="A116" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G116" t="s">
         <v>9</v>
@@ -2445,7 +2439,7 @@
     </row>
     <row r="117" spans="1:8">
       <c r="A117" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G117" t="s">
         <v>9</v>
@@ -2456,7 +2450,7 @@
     </row>
     <row r="118" spans="1:8">
       <c r="A118" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G118" t="s">
         <v>9</v>
@@ -2467,7 +2461,7 @@
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G119" t="s">
         <v>9</v>
@@ -2478,7 +2472,7 @@
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G120" t="s">
         <v>9</v>
@@ -2489,7 +2483,7 @@
     </row>
     <row r="121" spans="1:8">
       <c r="A121" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G121" t="s">
         <v>9</v>
@@ -2500,7 +2494,7 @@
     </row>
     <row r="122" spans="1:8">
       <c r="A122" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G122" t="s">
         <v>9</v>
@@ -2511,7 +2505,7 @@
     </row>
     <row r="123" spans="1:8">
       <c r="A123" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G123" t="s">
         <v>9</v>
@@ -2522,7 +2516,7 @@
     </row>
     <row r="124" spans="1:8">
       <c r="A124" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G124" t="s">
         <v>9</v>
@@ -2533,7 +2527,7 @@
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G125" t="s">
         <v>9</v>
@@ -2544,7 +2538,7 @@
     </row>
     <row r="126" spans="1:8">
       <c r="A126" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G126" t="s">
         <v>9</v>
@@ -2555,7 +2549,7 @@
     </row>
     <row r="127" spans="1:8">
       <c r="A127" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G127" t="s">
         <v>9</v>
@@ -2566,7 +2560,7 @@
     </row>
     <row r="128" spans="1:8">
       <c r="A128" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G128" t="s">
         <v>9</v>
@@ -2577,7 +2571,7 @@
     </row>
     <row r="129" spans="1:8">
       <c r="A129" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G129" t="s">
         <v>9</v>
@@ -2588,7 +2582,7 @@
     </row>
     <row r="130" spans="1:8">
       <c r="A130" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G130" t="s">
         <v>9</v>
@@ -2599,7 +2593,7 @@
     </row>
     <row r="131" spans="1:8">
       <c r="A131" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G131" t="s">
         <v>9</v>
@@ -2610,7 +2604,7 @@
     </row>
     <row r="132" spans="1:8">
       <c r="A132" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G132" t="s">
         <v>9</v>
@@ -2621,7 +2615,7 @@
     </row>
     <row r="133" spans="1:8">
       <c r="A133" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G133" t="s">
         <v>9</v>
@@ -2632,7 +2626,7 @@
     </row>
     <row r="134" spans="1:8">
       <c r="A134" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G134" t="s">
         <v>9</v>
@@ -2643,7 +2637,7 @@
     </row>
     <row r="135" spans="1:8">
       <c r="A135" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G135" t="s">
         <v>9</v>
@@ -2654,7 +2648,7 @@
     </row>
     <row r="136" spans="1:8">
       <c r="A136" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G136" t="s">
         <v>9</v>
@@ -2665,7 +2659,7 @@
     </row>
     <row r="137" spans="1:8">
       <c r="A137" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G137" t="s">
         <v>9</v>
@@ -2676,7 +2670,7 @@
     </row>
     <row r="138" spans="1:8">
       <c r="A138" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G138" t="s">
         <v>9</v>
@@ -2687,7 +2681,7 @@
     </row>
     <row r="139" spans="1:8">
       <c r="A139" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G139" t="s">
         <v>9</v>
@@ -2698,7 +2692,7 @@
     </row>
     <row r="140" spans="1:8">
       <c r="A140" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G140" t="s">
         <v>9</v>
@@ -2709,7 +2703,7 @@
     </row>
     <row r="141" spans="1:8">
       <c r="A141" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G141" t="s">
         <v>9</v>
@@ -2720,7 +2714,7 @@
     </row>
     <row r="142" spans="1:8">
       <c r="A142" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G142" t="s">
         <v>9</v>
@@ -2731,7 +2725,7 @@
     </row>
     <row r="143" spans="1:8">
       <c r="A143" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G143" t="s">
         <v>9</v>
@@ -2742,7 +2736,7 @@
     </row>
     <row r="144" spans="1:8">
       <c r="A144" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G144" t="s">
         <v>9</v>
@@ -2753,7 +2747,7 @@
     </row>
     <row r="145" spans="1:8">
       <c r="A145" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G145" t="s">
         <v>9</v>
@@ -2764,7 +2758,7 @@
     </row>
     <row r="146" spans="1:8">
       <c r="A146" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G146" t="s">
         <v>9</v>
@@ -2775,7 +2769,7 @@
     </row>
     <row r="147" spans="1:8">
       <c r="A147" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G147" t="s">
         <v>9</v>
@@ -2786,7 +2780,7 @@
     </row>
     <row r="148" spans="1:8">
       <c r="A148" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G148" t="s">
         <v>9</v>
@@ -2797,7 +2791,7 @@
     </row>
     <row r="149" spans="1:8">
       <c r="A149" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G149" t="s">
         <v>9</v>
@@ -2808,7 +2802,7 @@
     </row>
     <row r="150" spans="1:8">
       <c r="A150" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G150" t="s">
         <v>9</v>
@@ -2819,7 +2813,7 @@
     </row>
     <row r="151" spans="1:8">
       <c r="A151" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G151" t="s">
         <v>9</v>
@@ -2830,7 +2824,7 @@
     </row>
     <row r="152" spans="1:8">
       <c r="A152" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G152" t="s">
         <v>9</v>
@@ -2841,7 +2835,7 @@
     </row>
     <row r="153" spans="1:8">
       <c r="A153" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G153" t="s">
         <v>9</v>
@@ -2852,7 +2846,7 @@
     </row>
     <row r="154" spans="1:8">
       <c r="A154" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G154" t="s">
         <v>9</v>
@@ -2863,7 +2857,7 @@
     </row>
     <row r="155" spans="1:8">
       <c r="A155" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G155" t="s">
         <v>9</v>
@@ -2874,7 +2868,7 @@
     </row>
     <row r="156" spans="1:8">
       <c r="A156" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G156" t="s">
         <v>9</v>
@@ -2885,7 +2879,7 @@
     </row>
     <row r="157" spans="1:8">
       <c r="A157" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G157" t="s">
         <v>9</v>
@@ -2896,7 +2890,7 @@
     </row>
     <row r="158" spans="1:8">
       <c r="A158" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G158" t="s">
         <v>9</v>
@@ -2907,7 +2901,7 @@
     </row>
     <row r="159" spans="1:8">
       <c r="A159" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G159" t="s">
         <v>9</v>
@@ -2918,7 +2912,7 @@
     </row>
     <row r="160" spans="1:8">
       <c r="A160" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G160" t="s">
         <v>9</v>
@@ -2929,7 +2923,7 @@
     </row>
     <row r="161" spans="1:8">
       <c r="A161" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G161" t="s">
         <v>9</v>
@@ -2940,7 +2934,7 @@
     </row>
     <row r="162" spans="1:8">
       <c r="A162" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G162" t="s">
         <v>9</v>
@@ -2951,7 +2945,7 @@
     </row>
     <row r="163" spans="1:8">
       <c r="A163" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G163" t="s">
         <v>9</v>
@@ -2962,7 +2956,7 @@
     </row>
     <row r="164" spans="1:8">
       <c r="A164" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G164" t="s">
         <v>9</v>
@@ -2973,7 +2967,7 @@
     </row>
     <row r="165" spans="1:8">
       <c r="A165" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G165" t="s">
         <v>9</v>
@@ -2984,7 +2978,7 @@
     </row>
     <row r="166" spans="1:8">
       <c r="A166" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G166" t="s">
         <v>9</v>
@@ -2995,7 +2989,7 @@
     </row>
     <row r="167" spans="1:8">
       <c r="A167" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G167" t="s">
         <v>9</v>
@@ -3006,7 +3000,7 @@
     </row>
     <row r="168" spans="1:8">
       <c r="A168" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G168" t="s">
         <v>9</v>
@@ -3017,7 +3011,7 @@
     </row>
     <row r="169" spans="1:8">
       <c r="A169" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G169" t="s">
         <v>9</v>
@@ -3028,7 +3022,7 @@
     </row>
     <row r="170" spans="1:8">
       <c r="A170" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G170" t="s">
         <v>9</v>
@@ -3039,7 +3033,7 @@
     </row>
     <row r="171" spans="1:8">
       <c r="A171" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G171" t="s">
         <v>9</v>
@@ -3050,7 +3044,7 @@
     </row>
     <row r="172" spans="1:8">
       <c r="A172" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G172" t="s">
         <v>9</v>
@@ -3061,7 +3055,7 @@
     </row>
     <row r="173" spans="1:8">
       <c r="A173" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G173" t="s">
         <v>9</v>
@@ -3072,7 +3066,7 @@
     </row>
     <row r="174" spans="1:8">
       <c r="A174" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G174" t="s">
         <v>9</v>
@@ -3083,7 +3077,7 @@
     </row>
     <row r="175" spans="1:8">
       <c r="A175" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G175" t="s">
         <v>9</v>
@@ -3094,7 +3088,7 @@
     </row>
     <row r="176" spans="1:8">
       <c r="A176" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G176" t="s">
         <v>9</v>
@@ -3105,7 +3099,7 @@
     </row>
     <row r="177" spans="1:8">
       <c r="A177" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G177" t="s">
         <v>9</v>
@@ -3116,7 +3110,7 @@
     </row>
     <row r="178" spans="1:8">
       <c r="A178" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G178" t="s">
         <v>9</v>
@@ -3127,7 +3121,7 @@
     </row>
     <row r="179" spans="1:8">
       <c r="A179" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G179" t="s">
         <v>9</v>
@@ -3138,7 +3132,7 @@
     </row>
     <row r="180" spans="1:8">
       <c r="A180" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G180" t="s">
         <v>9</v>
@@ -3149,7 +3143,7 @@
     </row>
     <row r="181" spans="1:8">
       <c r="A181" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G181" t="s">
         <v>9</v>
@@ -3160,7 +3154,7 @@
     </row>
     <row r="182" spans="1:8">
       <c r="A182" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G182" t="s">
         <v>9</v>
@@ -3171,7 +3165,7 @@
     </row>
     <row r="183" spans="1:8">
       <c r="A183" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G183" t="s">
         <v>9</v>
@@ -3182,7 +3176,7 @@
     </row>
     <row r="184" spans="1:8">
       <c r="A184" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G184" t="s">
         <v>9</v>
@@ -3193,7 +3187,7 @@
     </row>
     <row r="185" spans="1:8">
       <c r="A185" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G185" t="s">
         <v>9</v>
@@ -3204,7 +3198,7 @@
     </row>
     <row r="186" spans="1:8">
       <c r="A186" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G186" t="s">
         <v>9</v>
@@ -3215,7 +3209,7 @@
     </row>
     <row r="187" spans="1:8">
       <c r="A187" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G187" t="s">
         <v>9</v>
@@ -3226,7 +3220,7 @@
     </row>
     <row r="188" spans="1:8">
       <c r="A188" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G188" t="s">
         <v>9</v>
@@ -3237,7 +3231,7 @@
     </row>
     <row r="189" spans="1:8">
       <c r="A189" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G189" t="s">
         <v>9</v>
@@ -3248,7 +3242,7 @@
     </row>
     <row r="190" spans="1:8">
       <c r="A190" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G190" t="s">
         <v>9</v>
@@ -3259,7 +3253,7 @@
     </row>
     <row r="191" spans="1:8">
       <c r="A191" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G191" t="s">
         <v>9</v>
@@ -3270,7 +3264,7 @@
     </row>
     <row r="192" spans="1:8">
       <c r="A192" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G192" t="s">
         <v>9</v>
@@ -3281,7 +3275,7 @@
     </row>
     <row r="193" spans="1:8">
       <c r="A193" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G193" t="s">
         <v>9</v>
@@ -3292,7 +3286,7 @@
     </row>
     <row r="194" spans="1:8">
       <c r="A194" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G194" t="s">
         <v>9</v>
@@ -3303,7 +3297,7 @@
     </row>
     <row r="195" spans="1:8">
       <c r="A195" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G195" t="s">
         <v>9</v>
@@ -3314,7 +3308,7 @@
     </row>
     <row r="196" spans="1:8">
       <c r="A196" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G196" t="s">
         <v>9</v>
@@ -3325,7 +3319,7 @@
     </row>
     <row r="197" spans="1:8">
       <c r="A197" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G197" t="s">
         <v>9</v>
@@ -3336,7 +3330,7 @@
     </row>
     <row r="198" spans="1:8">
       <c r="A198" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G198" t="s">
         <v>9</v>
@@ -3347,7 +3341,7 @@
     </row>
     <row r="199" spans="1:8">
       <c r="A199" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G199" t="s">
         <v>9</v>
@@ -3358,7 +3352,7 @@
     </row>
     <row r="200" spans="1:8">
       <c r="A200" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G200" t="s">
         <v>9</v>
@@ -3369,7 +3363,7 @@
     </row>
     <row r="201" spans="1:8">
       <c r="A201" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G201" t="s">
         <v>9</v>
@@ -3380,7 +3374,7 @@
     </row>
     <row r="202" spans="1:8">
       <c r="A202" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G202" t="s">
         <v>9</v>
@@ -3391,7 +3385,7 @@
     </row>
     <row r="203" spans="1:8">
       <c r="A203" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G203" t="s">
         <v>9</v>
@@ -3402,7 +3396,7 @@
     </row>
     <row r="204" spans="1:8">
       <c r="A204" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G204" t="s">
         <v>9</v>
@@ -3413,7 +3407,7 @@
     </row>
     <row r="205" spans="1:8">
       <c r="A205" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G205" t="s">
         <v>9</v>
@@ -3424,7 +3418,7 @@
     </row>
     <row r="206" spans="1:8">
       <c r="A206" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G206" t="s">
         <v>9</v>
@@ -3435,7 +3429,7 @@
     </row>
     <row r="207" spans="1:8">
       <c r="A207" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G207" t="s">
         <v>9</v>
@@ -3446,7 +3440,7 @@
     </row>
     <row r="208" spans="1:8">
       <c r="A208" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G208" t="s">
         <v>9</v>
@@ -3457,7 +3451,7 @@
     </row>
     <row r="209" spans="1:8">
       <c r="A209" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G209" t="s">
         <v>9</v>
@@ -3468,7 +3462,7 @@
     </row>
     <row r="210" spans="1:8">
       <c r="A210" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G210" t="s">
         <v>9</v>
@@ -3479,7 +3473,7 @@
     </row>
     <row r="211" spans="1:8">
       <c r="A211" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G211" t="s">
         <v>9</v>
@@ -3490,7 +3484,7 @@
     </row>
     <row r="212" spans="1:8">
       <c r="A212" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G212" t="s">
         <v>9</v>
@@ -3501,7 +3495,7 @@
     </row>
     <row r="213" spans="1:8">
       <c r="A213" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G213" t="s">
         <v>9</v>
@@ -3512,7 +3506,7 @@
     </row>
     <row r="214" spans="1:8">
       <c r="A214" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G214" t="s">
         <v>9</v>
@@ -3523,7 +3517,7 @@
     </row>
     <row r="215" spans="1:8">
       <c r="A215" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G215" t="s">
         <v>9</v>
@@ -3534,7 +3528,7 @@
     </row>
     <row r="216" spans="1:8">
       <c r="A216" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G216" t="s">
         <v>9</v>
@@ -3545,7 +3539,7 @@
     </row>
     <row r="217" spans="1:8">
       <c r="A217" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G217" t="s">
         <v>9</v>
@@ -3556,7 +3550,7 @@
     </row>
     <row r="218" spans="1:8">
       <c r="A218" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G218" t="s">
         <v>9</v>
@@ -3567,7 +3561,7 @@
     </row>
     <row r="219" spans="1:8">
       <c r="A219" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G219" t="s">
         <v>9</v>
@@ -3578,7 +3572,7 @@
     </row>
     <row r="220" spans="1:8">
       <c r="A220" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G220" t="s">
         <v>9</v>
@@ -3589,7 +3583,7 @@
     </row>
     <row r="221" spans="1:8">
       <c r="A221" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G221" t="s">
         <v>9</v>
@@ -3600,7 +3594,7 @@
     </row>
     <row r="222" spans="1:8">
       <c r="A222" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G222" t="s">
         <v>9</v>
@@ -3611,7 +3605,7 @@
     </row>
     <row r="223" spans="1:8">
       <c r="A223" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G223" t="s">
         <v>9</v>
@@ -3622,7 +3616,7 @@
     </row>
     <row r="224" spans="1:8">
       <c r="A224" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G224" t="s">
         <v>9</v>
@@ -3633,7 +3627,7 @@
     </row>
     <row r="225" spans="1:8">
       <c r="A225" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G225" t="s">
         <v>9</v>
@@ -3644,7 +3638,7 @@
     </row>
     <row r="226" spans="1:8">
       <c r="A226" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G226" t="s">
         <v>9</v>
@@ -3655,7 +3649,7 @@
     </row>
     <row r="227" spans="1:8">
       <c r="A227" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G227" t="s">
         <v>9</v>
@@ -3666,7 +3660,7 @@
     </row>
     <row r="228" spans="1:8">
       <c r="A228" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G228" t="s">
         <v>9</v>
@@ -3677,7 +3671,7 @@
     </row>
     <row r="229" spans="1:8">
       <c r="A229" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G229" t="s">
         <v>9</v>
@@ -3688,7 +3682,7 @@
     </row>
     <row r="230" spans="1:8">
       <c r="A230" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G230" t="s">
         <v>9</v>
@@ -3699,7 +3693,7 @@
     </row>
     <row r="231" spans="1:8">
       <c r="A231" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G231" t="s">
         <v>9</v>
@@ -3710,7 +3704,7 @@
     </row>
     <row r="232" spans="1:8">
       <c r="A232" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G232" t="s">
         <v>9</v>
@@ -3721,7 +3715,7 @@
     </row>
     <row r="233" spans="1:8">
       <c r="A233" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G233" t="s">
         <v>9</v>
@@ -3732,7 +3726,7 @@
     </row>
     <row r="234" spans="1:8">
       <c r="A234" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G234" t="s">
         <v>9</v>
@@ -3743,7 +3737,7 @@
     </row>
     <row r="235" spans="1:8">
       <c r="A235" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G235" t="s">
         <v>9</v>
@@ -3754,7 +3748,7 @@
     </row>
     <row r="236" spans="1:8">
       <c r="A236" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G236" t="s">
         <v>9</v>
@@ -3765,7 +3759,7 @@
     </row>
     <row r="237" spans="1:8">
       <c r="A237" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G237" t="s">
         <v>9</v>
@@ -3776,7 +3770,7 @@
     </row>
     <row r="238" spans="1:8">
       <c r="A238" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G238" t="s">
         <v>9</v>
@@ -3787,7 +3781,7 @@
     </row>
     <row r="239" spans="1:8">
       <c r="A239" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G239" t="s">
         <v>9</v>
@@ -3798,7 +3792,7 @@
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G240" t="s">
         <v>9</v>
@@ -3809,7 +3803,7 @@
     </row>
     <row r="241" spans="1:8">
       <c r="A241" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G241" t="s">
         <v>9</v>
@@ -3820,7 +3814,7 @@
     </row>
     <row r="242" spans="1:8">
       <c r="A242" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G242" t="s">
         <v>9</v>
@@ -3831,7 +3825,7 @@
     </row>
     <row r="243" spans="1:8">
       <c r="A243" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G243" t="s">
         <v>9</v>
@@ -3842,7 +3836,7 @@
     </row>
     <row r="244" spans="1:8">
       <c r="A244" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G244" t="s">
         <v>9</v>
@@ -3853,7 +3847,7 @@
     </row>
     <row r="245" spans="1:8">
       <c r="A245" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G245" t="s">
         <v>9</v>
@@ -3864,7 +3858,7 @@
     </row>
     <row r="246" spans="1:8">
       <c r="A246" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G246" t="s">
         <v>9</v>
@@ -3875,7 +3869,7 @@
     </row>
     <row r="247" spans="1:8">
       <c r="A247" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G247" t="s">
         <v>9</v>
@@ -3886,7 +3880,7 @@
     </row>
     <row r="248" spans="1:8">
       <c r="A248" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G248" t="s">
         <v>9</v>
@@ -3897,7 +3891,7 @@
     </row>
     <row r="249" spans="1:8">
       <c r="A249" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G249" t="s">
         <v>9</v>
@@ -3908,7 +3902,7 @@
     </row>
     <row r="250" spans="1:8">
       <c r="A250" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G250" t="s">
         <v>9</v>
@@ -3919,7 +3913,7 @@
     </row>
     <row r="251" spans="1:8">
       <c r="A251" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G251" t="s">
         <v>9</v>
@@ -3930,7 +3924,7 @@
     </row>
     <row r="252" spans="1:8">
       <c r="A252" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G252" t="s">
         <v>9</v>
@@ -3941,7 +3935,7 @@
     </row>
     <row r="253" spans="1:8">
       <c r="A253" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G253" t="s">
         <v>9</v>
@@ -3952,7 +3946,7 @@
     </row>
     <row r="254" spans="1:8">
       <c r="A254" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G254" t="s">
         <v>9</v>
@@ -3963,7 +3957,7 @@
     </row>
     <row r="255" spans="1:8">
       <c r="A255" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G255" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
fixed automatic excel column getter
</commit_message>
<xml_diff>
--- a/stationsinformation.xlsx
+++ b/stationsinformation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="265">
   <si>
     <t>Device</t>
   </si>
@@ -1177,7 +1177,7 @@
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1188,7 +1188,7 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H3" t="s">
         <v>9</v>
@@ -1199,7 +1199,7 @@
         <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" t="s">
         <v>9</v>
@@ -1210,7 +1210,7 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H5" t="s">
         <v>9</v>
@@ -1221,7 +1221,7 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
         <v>9</v>
@@ -1232,7 +1232,7 @@
         <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H7" t="s">
         <v>9</v>
@@ -1243,7 +1243,7 @@
         <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H8" t="s">
         <v>9</v>
@@ -1254,7 +1254,7 @@
         <v>18</v>
       </c>
       <c r="G9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H9" t="s">
         <v>9</v>
@@ -1265,7 +1265,7 @@
         <v>19</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H10" t="s">
         <v>9</v>
@@ -1276,7 +1276,7 @@
         <v>20</v>
       </c>
       <c r="G11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H11" t="s">
         <v>9</v>
@@ -1287,7 +1287,7 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H12" t="s">
         <v>9</v>
@@ -1298,7 +1298,7 @@
         <v>22</v>
       </c>
       <c r="G13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H13" t="s">
         <v>9</v>
@@ -1309,7 +1309,7 @@
         <v>23</v>
       </c>
       <c r="G14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H14" t="s">
         <v>9</v>
@@ -1320,7 +1320,7 @@
         <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H15" t="s">
         <v>9</v>
@@ -1331,7 +1331,7 @@
         <v>25</v>
       </c>
       <c r="G16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H16" t="s">
         <v>9</v>
@@ -1342,7 +1342,7 @@
         <v>26</v>
       </c>
       <c r="G17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H17" t="s">
         <v>9</v>
@@ -1353,7 +1353,7 @@
         <v>27</v>
       </c>
       <c r="G18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H18" t="s">
         <v>9</v>
@@ -1364,7 +1364,7 @@
         <v>28</v>
       </c>
       <c r="G19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H19" t="s">
         <v>9</v>
@@ -1375,7 +1375,7 @@
         <v>29</v>
       </c>
       <c r="G20" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H20" t="s">
         <v>9</v>
@@ -1386,7 +1386,7 @@
         <v>30</v>
       </c>
       <c r="G21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H21" t="s">
         <v>9</v>
@@ -1397,7 +1397,7 @@
         <v>31</v>
       </c>
       <c r="G22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H22" t="s">
         <v>9</v>
@@ -1408,7 +1408,7 @@
         <v>32</v>
       </c>
       <c r="G23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23" t="s">
         <v>9</v>
@@ -1419,7 +1419,7 @@
         <v>33</v>
       </c>
       <c r="G24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H24" t="s">
         <v>9</v>
@@ -1430,7 +1430,7 @@
         <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H25" t="s">
         <v>9</v>
@@ -1441,7 +1441,7 @@
         <v>35</v>
       </c>
       <c r="G26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H26" t="s">
         <v>9</v>
@@ -1452,7 +1452,7 @@
         <v>36</v>
       </c>
       <c r="G27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H27" t="s">
         <v>9</v>
@@ -1463,7 +1463,7 @@
         <v>37</v>
       </c>
       <c r="G28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H28" t="s">
         <v>9</v>
@@ -1474,7 +1474,7 @@
         <v>38</v>
       </c>
       <c r="G29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H29" t="s">
         <v>9</v>
@@ -1485,7 +1485,7 @@
         <v>39</v>
       </c>
       <c r="G30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H30" t="s">
         <v>9</v>
@@ -1496,7 +1496,7 @@
         <v>40</v>
       </c>
       <c r="G31" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H31" t="s">
         <v>9</v>
@@ -1507,7 +1507,7 @@
         <v>41</v>
       </c>
       <c r="G32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H32" t="s">
         <v>9</v>
@@ -1518,7 +1518,7 @@
         <v>42</v>
       </c>
       <c r="G33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H33" t="s">
         <v>9</v>
@@ -1529,7 +1529,7 @@
         <v>43</v>
       </c>
       <c r="G34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H34" t="s">
         <v>9</v>
@@ -1540,7 +1540,7 @@
         <v>44</v>
       </c>
       <c r="G35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H35" t="s">
         <v>9</v>
@@ -1551,7 +1551,7 @@
         <v>45</v>
       </c>
       <c r="G36" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H36" t="s">
         <v>9</v>
@@ -1562,7 +1562,7 @@
         <v>46</v>
       </c>
       <c r="G37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H37" t="s">
         <v>9</v>
@@ -1573,7 +1573,7 @@
         <v>47</v>
       </c>
       <c r="G38" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H38" t="s">
         <v>9</v>
@@ -1584,7 +1584,7 @@
         <v>48</v>
       </c>
       <c r="G39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H39" t="s">
         <v>9</v>
@@ -1595,7 +1595,7 @@
         <v>49</v>
       </c>
       <c r="G40" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H40" t="s">
         <v>9</v>
@@ -1606,7 +1606,7 @@
         <v>50</v>
       </c>
       <c r="G41" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H41" t="s">
         <v>9</v>
@@ -1617,7 +1617,7 @@
         <v>51</v>
       </c>
       <c r="G42" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H42" t="s">
         <v>9</v>
@@ -1628,7 +1628,7 @@
         <v>52</v>
       </c>
       <c r="G43" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H43" t="s">
         <v>9</v>
@@ -1639,7 +1639,7 @@
         <v>53</v>
       </c>
       <c r="G44" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H44" t="s">
         <v>9</v>
@@ -1650,7 +1650,7 @@
         <v>54</v>
       </c>
       <c r="G45" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H45" t="s">
         <v>9</v>
@@ -1661,7 +1661,7 @@
         <v>55</v>
       </c>
       <c r="G46" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H46" t="s">
         <v>9</v>
@@ -1672,7 +1672,7 @@
         <v>56</v>
       </c>
       <c r="G47" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H47" t="s">
         <v>9</v>
@@ -1683,7 +1683,7 @@
         <v>57</v>
       </c>
       <c r="G48" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H48" t="s">
         <v>9</v>
@@ -1694,7 +1694,7 @@
         <v>58</v>
       </c>
       <c r="G49" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H49" t="s">
         <v>9</v>
@@ -1705,7 +1705,7 @@
         <v>59</v>
       </c>
       <c r="G50" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H50" t="s">
         <v>9</v>
@@ -1716,7 +1716,7 @@
         <v>60</v>
       </c>
       <c r="G51" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H51" t="s">
         <v>9</v>
@@ -1727,7 +1727,7 @@
         <v>61</v>
       </c>
       <c r="G52" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H52" t="s">
         <v>9</v>
@@ -1738,7 +1738,7 @@
         <v>62</v>
       </c>
       <c r="G53" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H53" t="s">
         <v>9</v>
@@ -1749,7 +1749,7 @@
         <v>63</v>
       </c>
       <c r="G54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H54" t="s">
         <v>9</v>
@@ -1760,7 +1760,7 @@
         <v>64</v>
       </c>
       <c r="G55" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H55" t="s">
         <v>9</v>
@@ -1771,7 +1771,7 @@
         <v>65</v>
       </c>
       <c r="G56" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H56" t="s">
         <v>9</v>
@@ -1782,7 +1782,7 @@
         <v>66</v>
       </c>
       <c r="G57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H57" t="s">
         <v>9</v>
@@ -1793,7 +1793,7 @@
         <v>67</v>
       </c>
       <c r="G58" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H58" t="s">
         <v>9</v>
@@ -1804,7 +1804,7 @@
         <v>68</v>
       </c>
       <c r="G59" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H59" t="s">
         <v>9</v>
@@ -1815,7 +1815,7 @@
         <v>69</v>
       </c>
       <c r="G60" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H60" t="s">
         <v>9</v>
@@ -1826,7 +1826,7 @@
         <v>70</v>
       </c>
       <c r="G61" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H61" t="s">
         <v>9</v>
@@ -1837,7 +1837,7 @@
         <v>71</v>
       </c>
       <c r="G62" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H62" t="s">
         <v>9</v>
@@ -1848,7 +1848,7 @@
         <v>72</v>
       </c>
       <c r="G63" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H63" t="s">
         <v>9</v>
@@ -1859,7 +1859,7 @@
         <v>73</v>
       </c>
       <c r="G64" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H64" t="s">
         <v>9</v>
@@ -1870,7 +1870,7 @@
         <v>74</v>
       </c>
       <c r="G65" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H65" t="s">
         <v>9</v>
@@ -1881,7 +1881,7 @@
         <v>75</v>
       </c>
       <c r="G66" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H66" t="s">
         <v>9</v>
@@ -1892,7 +1892,7 @@
         <v>76</v>
       </c>
       <c r="G67" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H67" t="s">
         <v>9</v>
@@ -1903,7 +1903,7 @@
         <v>77</v>
       </c>
       <c r="G68" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H68" t="s">
         <v>9</v>
@@ -1914,7 +1914,7 @@
         <v>78</v>
       </c>
       <c r="G69" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H69" t="s">
         <v>9</v>
@@ -1925,7 +1925,7 @@
         <v>79</v>
       </c>
       <c r="G70" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H70" t="s">
         <v>9</v>
@@ -1936,7 +1936,7 @@
         <v>80</v>
       </c>
       <c r="G71" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H71" t="s">
         <v>9</v>
@@ -1947,7 +1947,7 @@
         <v>81</v>
       </c>
       <c r="G72" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H72" t="s">
         <v>9</v>
@@ -1958,7 +1958,7 @@
         <v>82</v>
       </c>
       <c r="G73" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H73" t="s">
         <v>9</v>
@@ -1969,7 +1969,7 @@
         <v>83</v>
       </c>
       <c r="G74" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H74" t="s">
         <v>9</v>
@@ -1980,7 +1980,7 @@
         <v>84</v>
       </c>
       <c r="G75" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H75" t="s">
         <v>9</v>
@@ -1991,7 +1991,7 @@
         <v>85</v>
       </c>
       <c r="G76" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H76" t="s">
         <v>9</v>
@@ -2002,7 +2002,7 @@
         <v>86</v>
       </c>
       <c r="G77" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H77" t="s">
         <v>9</v>
@@ -2013,7 +2013,7 @@
         <v>87</v>
       </c>
       <c r="G78" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H78" t="s">
         <v>9</v>
@@ -2024,7 +2024,7 @@
         <v>88</v>
       </c>
       <c r="G79" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H79" t="s">
         <v>9</v>
@@ -2035,7 +2035,7 @@
         <v>89</v>
       </c>
       <c r="G80" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H80" t="s">
         <v>9</v>
@@ -2046,7 +2046,7 @@
         <v>90</v>
       </c>
       <c r="G81" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H81" t="s">
         <v>9</v>
@@ -2057,7 +2057,7 @@
         <v>91</v>
       </c>
       <c r="G82" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H82" t="s">
         <v>9</v>
@@ -2068,7 +2068,7 @@
         <v>92</v>
       </c>
       <c r="G83" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H83" t="s">
         <v>9</v>
@@ -2079,7 +2079,7 @@
         <v>93</v>
       </c>
       <c r="G84" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H84" t="s">
         <v>9</v>
@@ -2090,7 +2090,7 @@
         <v>94</v>
       </c>
       <c r="G85" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H85" t="s">
         <v>9</v>
@@ -2101,7 +2101,7 @@
         <v>95</v>
       </c>
       <c r="G86" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H86" t="s">
         <v>9</v>
@@ -2112,7 +2112,7 @@
         <v>96</v>
       </c>
       <c r="G87" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H87" t="s">
         <v>9</v>
@@ -2123,7 +2123,7 @@
         <v>97</v>
       </c>
       <c r="G88" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H88" t="s">
         <v>9</v>
@@ -2134,7 +2134,7 @@
         <v>98</v>
       </c>
       <c r="G89" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H89" t="s">
         <v>9</v>
@@ -2145,7 +2145,7 @@
         <v>99</v>
       </c>
       <c r="G90" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H90" t="s">
         <v>9</v>
@@ -2156,7 +2156,7 @@
         <v>100</v>
       </c>
       <c r="G91" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H91" t="s">
         <v>9</v>
@@ -2167,7 +2167,7 @@
         <v>101</v>
       </c>
       <c r="G92" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H92" t="s">
         <v>9</v>
@@ -2178,7 +2178,7 @@
         <v>102</v>
       </c>
       <c r="G93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H93" t="s">
         <v>9</v>
@@ -2189,7 +2189,7 @@
         <v>103</v>
       </c>
       <c r="G94" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H94" t="s">
         <v>9</v>
@@ -2200,7 +2200,7 @@
         <v>104</v>
       </c>
       <c r="G95" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H95" t="s">
         <v>9</v>
@@ -2211,7 +2211,7 @@
         <v>105</v>
       </c>
       <c r="G96" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H96" t="s">
         <v>9</v>
@@ -2222,7 +2222,7 @@
         <v>106</v>
       </c>
       <c r="G97" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H97" t="s">
         <v>9</v>
@@ -2233,7 +2233,7 @@
         <v>107</v>
       </c>
       <c r="G98" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H98" t="s">
         <v>9</v>
@@ -2244,7 +2244,7 @@
         <v>108</v>
       </c>
       <c r="G99" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H99" t="s">
         <v>9</v>
@@ -2255,7 +2255,7 @@
         <v>109</v>
       </c>
       <c r="G100" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H100" t="s">
         <v>9</v>
@@ -2266,7 +2266,7 @@
         <v>110</v>
       </c>
       <c r="G101" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H101" t="s">
         <v>9</v>
@@ -2277,7 +2277,7 @@
         <v>111</v>
       </c>
       <c r="G102" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H102" t="s">
         <v>9</v>
@@ -2288,7 +2288,7 @@
         <v>112</v>
       </c>
       <c r="G103" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H103" t="s">
         <v>9</v>
@@ -2299,7 +2299,7 @@
         <v>113</v>
       </c>
       <c r="G104" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H104" t="s">
         <v>9</v>
@@ -2310,7 +2310,7 @@
         <v>114</v>
       </c>
       <c r="G105" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H105" t="s">
         <v>9</v>
@@ -2321,7 +2321,7 @@
         <v>115</v>
       </c>
       <c r="G106" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H106" t="s">
         <v>9</v>
@@ -2332,7 +2332,7 @@
         <v>116</v>
       </c>
       <c r="G107" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H107" t="s">
         <v>9</v>
@@ -2343,7 +2343,7 @@
         <v>117</v>
       </c>
       <c r="G108" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H108" t="s">
         <v>9</v>
@@ -2354,7 +2354,7 @@
         <v>118</v>
       </c>
       <c r="G109" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H109" t="s">
         <v>9</v>
@@ -2365,7 +2365,7 @@
         <v>119</v>
       </c>
       <c r="G110" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H110" t="s">
         <v>9</v>
@@ -2376,7 +2376,7 @@
         <v>120</v>
       </c>
       <c r="G111" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H111" t="s">
         <v>9</v>
@@ -2387,7 +2387,7 @@
         <v>121</v>
       </c>
       <c r="G112" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H112" t="s">
         <v>9</v>
@@ -2398,7 +2398,7 @@
         <v>122</v>
       </c>
       <c r="G113" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H113" t="s">
         <v>9</v>
@@ -2409,7 +2409,7 @@
         <v>123</v>
       </c>
       <c r="G114" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H114" t="s">
         <v>9</v>
@@ -2420,7 +2420,7 @@
         <v>124</v>
       </c>
       <c r="G115" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H115" t="s">
         <v>9</v>
@@ -2431,7 +2431,7 @@
         <v>125</v>
       </c>
       <c r="G116" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H116" t="s">
         <v>9</v>
@@ -2442,7 +2442,7 @@
         <v>126</v>
       </c>
       <c r="G117" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H117" t="s">
         <v>9</v>
@@ -2453,7 +2453,7 @@
         <v>127</v>
       </c>
       <c r="G118" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H118" t="s">
         <v>9</v>
@@ -2464,7 +2464,7 @@
         <v>128</v>
       </c>
       <c r="G119" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H119" t="s">
         <v>9</v>
@@ -2475,7 +2475,7 @@
         <v>129</v>
       </c>
       <c r="G120" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H120" t="s">
         <v>9</v>
@@ -2486,7 +2486,7 @@
         <v>130</v>
       </c>
       <c r="G121" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H121" t="s">
         <v>9</v>
@@ -2497,7 +2497,7 @@
         <v>131</v>
       </c>
       <c r="G122" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H122" t="s">
         <v>9</v>
@@ -2508,7 +2508,7 @@
         <v>132</v>
       </c>
       <c r="G123" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H123" t="s">
         <v>9</v>
@@ -2519,7 +2519,7 @@
         <v>133</v>
       </c>
       <c r="G124" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H124" t="s">
         <v>9</v>
@@ -2530,7 +2530,7 @@
         <v>134</v>
       </c>
       <c r="G125" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H125" t="s">
         <v>9</v>
@@ -2541,7 +2541,7 @@
         <v>135</v>
       </c>
       <c r="G126" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H126" t="s">
         <v>9</v>
@@ -2552,7 +2552,7 @@
         <v>136</v>
       </c>
       <c r="G127" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H127" t="s">
         <v>9</v>
@@ -2563,7 +2563,7 @@
         <v>137</v>
       </c>
       <c r="G128" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H128" t="s">
         <v>9</v>
@@ -2574,7 +2574,7 @@
         <v>138</v>
       </c>
       <c r="G129" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H129" t="s">
         <v>9</v>
@@ -2585,7 +2585,7 @@
         <v>139</v>
       </c>
       <c r="G130" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H130" t="s">
         <v>9</v>
@@ -2596,7 +2596,7 @@
         <v>140</v>
       </c>
       <c r="G131" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H131" t="s">
         <v>9</v>
@@ -2607,7 +2607,7 @@
         <v>141</v>
       </c>
       <c r="G132" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H132" t="s">
         <v>9</v>
@@ -2618,7 +2618,7 @@
         <v>142</v>
       </c>
       <c r="G133" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H133" t="s">
         <v>9</v>
@@ -2629,7 +2629,7 @@
         <v>143</v>
       </c>
       <c r="G134" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H134" t="s">
         <v>9</v>
@@ -2640,7 +2640,7 @@
         <v>144</v>
       </c>
       <c r="G135" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H135" t="s">
         <v>9</v>
@@ -2651,7 +2651,7 @@
         <v>145</v>
       </c>
       <c r="G136" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H136" t="s">
         <v>9</v>
@@ -2662,7 +2662,7 @@
         <v>146</v>
       </c>
       <c r="G137" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H137" t="s">
         <v>9</v>
@@ -2673,7 +2673,7 @@
         <v>147</v>
       </c>
       <c r="G138" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H138" t="s">
         <v>9</v>
@@ -2684,7 +2684,7 @@
         <v>148</v>
       </c>
       <c r="G139" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H139" t="s">
         <v>9</v>
@@ -2695,7 +2695,7 @@
         <v>149</v>
       </c>
       <c r="G140" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H140" t="s">
         <v>9</v>
@@ -2706,7 +2706,7 @@
         <v>150</v>
       </c>
       <c r="G141" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H141" t="s">
         <v>9</v>
@@ -2717,7 +2717,7 @@
         <v>151</v>
       </c>
       <c r="G142" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H142" t="s">
         <v>9</v>
@@ -2728,7 +2728,7 @@
         <v>152</v>
       </c>
       <c r="G143" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H143" t="s">
         <v>9</v>
@@ -2739,7 +2739,7 @@
         <v>153</v>
       </c>
       <c r="G144" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H144" t="s">
         <v>9</v>
@@ -2750,7 +2750,7 @@
         <v>154</v>
       </c>
       <c r="G145" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H145" t="s">
         <v>9</v>
@@ -2761,7 +2761,7 @@
         <v>155</v>
       </c>
       <c r="G146" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H146" t="s">
         <v>9</v>
@@ -2772,7 +2772,7 @@
         <v>156</v>
       </c>
       <c r="G147" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H147" t="s">
         <v>9</v>
@@ -2783,7 +2783,7 @@
         <v>157</v>
       </c>
       <c r="G148" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H148" t="s">
         <v>9</v>
@@ -2794,7 +2794,7 @@
         <v>158</v>
       </c>
       <c r="G149" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H149" t="s">
         <v>9</v>
@@ -2805,7 +2805,7 @@
         <v>159</v>
       </c>
       <c r="G150" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H150" t="s">
         <v>9</v>
@@ -2816,7 +2816,7 @@
         <v>160</v>
       </c>
       <c r="G151" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H151" t="s">
         <v>9</v>
@@ -2827,7 +2827,7 @@
         <v>161</v>
       </c>
       <c r="G152" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H152" t="s">
         <v>9</v>
@@ -2838,7 +2838,7 @@
         <v>162</v>
       </c>
       <c r="G153" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H153" t="s">
         <v>9</v>
@@ -2849,7 +2849,7 @@
         <v>163</v>
       </c>
       <c r="G154" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H154" t="s">
         <v>9</v>
@@ -2860,7 +2860,7 @@
         <v>164</v>
       </c>
       <c r="G155" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H155" t="s">
         <v>9</v>
@@ -2871,7 +2871,7 @@
         <v>165</v>
       </c>
       <c r="G156" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H156" t="s">
         <v>9</v>
@@ -2882,7 +2882,7 @@
         <v>166</v>
       </c>
       <c r="G157" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H157" t="s">
         <v>9</v>
@@ -2893,7 +2893,7 @@
         <v>167</v>
       </c>
       <c r="G158" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H158" t="s">
         <v>9</v>
@@ -2904,7 +2904,7 @@
         <v>168</v>
       </c>
       <c r="G159" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H159" t="s">
         <v>9</v>
@@ -2915,7 +2915,7 @@
         <v>169</v>
       </c>
       <c r="G160" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H160" t="s">
         <v>9</v>
@@ -2926,7 +2926,7 @@
         <v>170</v>
       </c>
       <c r="G161" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H161" t="s">
         <v>9</v>
@@ -2937,7 +2937,7 @@
         <v>171</v>
       </c>
       <c r="G162" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H162" t="s">
         <v>9</v>
@@ -2948,7 +2948,7 @@
         <v>172</v>
       </c>
       <c r="G163" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H163" t="s">
         <v>9</v>
@@ -2959,7 +2959,7 @@
         <v>173</v>
       </c>
       <c r="G164" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H164" t="s">
         <v>9</v>
@@ -2970,7 +2970,7 @@
         <v>174</v>
       </c>
       <c r="G165" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H165" t="s">
         <v>9</v>
@@ -2981,7 +2981,7 @@
         <v>175</v>
       </c>
       <c r="G166" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H166" t="s">
         <v>9</v>
@@ -2992,7 +2992,7 @@
         <v>176</v>
       </c>
       <c r="G167" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H167" t="s">
         <v>9</v>
@@ -3003,7 +3003,7 @@
         <v>177</v>
       </c>
       <c r="G168" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H168" t="s">
         <v>9</v>
@@ -3014,7 +3014,7 @@
         <v>178</v>
       </c>
       <c r="G169" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H169" t="s">
         <v>9</v>
@@ -3025,7 +3025,7 @@
         <v>179</v>
       </c>
       <c r="G170" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H170" t="s">
         <v>9</v>
@@ -3036,7 +3036,7 @@
         <v>180</v>
       </c>
       <c r="G171" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H171" t="s">
         <v>9</v>
@@ -3047,7 +3047,7 @@
         <v>181</v>
       </c>
       <c r="G172" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H172" t="s">
         <v>9</v>
@@ -3058,7 +3058,7 @@
         <v>182</v>
       </c>
       <c r="G173" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H173" t="s">
         <v>9</v>
@@ -3069,7 +3069,7 @@
         <v>183</v>
       </c>
       <c r="G174" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H174" t="s">
         <v>9</v>
@@ -3080,7 +3080,7 @@
         <v>184</v>
       </c>
       <c r="G175" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H175" t="s">
         <v>9</v>
@@ -3091,7 +3091,7 @@
         <v>185</v>
       </c>
       <c r="G176" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H176" t="s">
         <v>9</v>
@@ -3102,7 +3102,7 @@
         <v>186</v>
       </c>
       <c r="G177" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H177" t="s">
         <v>9</v>
@@ -3113,7 +3113,7 @@
         <v>187</v>
       </c>
       <c r="G178" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H178" t="s">
         <v>9</v>
@@ -3124,7 +3124,7 @@
         <v>188</v>
       </c>
       <c r="G179" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H179" t="s">
         <v>9</v>
@@ -3135,7 +3135,7 @@
         <v>189</v>
       </c>
       <c r="G180" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H180" t="s">
         <v>9</v>
@@ -3146,7 +3146,7 @@
         <v>190</v>
       </c>
       <c r="G181" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H181" t="s">
         <v>9</v>
@@ -3157,7 +3157,7 @@
         <v>191</v>
       </c>
       <c r="G182" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H182" t="s">
         <v>9</v>
@@ -3168,7 +3168,7 @@
         <v>192</v>
       </c>
       <c r="G183" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H183" t="s">
         <v>9</v>
@@ -3179,7 +3179,7 @@
         <v>193</v>
       </c>
       <c r="G184" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H184" t="s">
         <v>9</v>
@@ -3190,7 +3190,7 @@
         <v>194</v>
       </c>
       <c r="G185" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H185" t="s">
         <v>9</v>
@@ -3201,7 +3201,7 @@
         <v>195</v>
       </c>
       <c r="G186" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H186" t="s">
         <v>9</v>
@@ -3212,7 +3212,7 @@
         <v>196</v>
       </c>
       <c r="G187" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H187" t="s">
         <v>9</v>
@@ -3223,7 +3223,7 @@
         <v>197</v>
       </c>
       <c r="G188" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H188" t="s">
         <v>9</v>
@@ -3234,7 +3234,7 @@
         <v>198</v>
       </c>
       <c r="G189" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H189" t="s">
         <v>9</v>
@@ -3245,7 +3245,7 @@
         <v>199</v>
       </c>
       <c r="G190" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H190" t="s">
         <v>9</v>
@@ -3256,7 +3256,7 @@
         <v>200</v>
       </c>
       <c r="G191" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H191" t="s">
         <v>9</v>
@@ -3267,7 +3267,7 @@
         <v>201</v>
       </c>
       <c r="G192" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H192" t="s">
         <v>9</v>
@@ -3278,7 +3278,7 @@
         <v>202</v>
       </c>
       <c r="G193" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H193" t="s">
         <v>9</v>
@@ -3289,7 +3289,7 @@
         <v>203</v>
       </c>
       <c r="G194" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H194" t="s">
         <v>9</v>
@@ -3300,7 +3300,7 @@
         <v>204</v>
       </c>
       <c r="G195" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H195" t="s">
         <v>9</v>
@@ -3311,7 +3311,7 @@
         <v>205</v>
       </c>
       <c r="G196" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H196" t="s">
         <v>9</v>
@@ -3322,7 +3322,7 @@
         <v>206</v>
       </c>
       <c r="G197" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H197" t="s">
         <v>9</v>
@@ -3333,7 +3333,7 @@
         <v>207</v>
       </c>
       <c r="G198" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H198" t="s">
         <v>9</v>
@@ -3344,7 +3344,7 @@
         <v>208</v>
       </c>
       <c r="G199" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H199" t="s">
         <v>9</v>
@@ -3355,7 +3355,7 @@
         <v>209</v>
       </c>
       <c r="G200" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H200" t="s">
         <v>9</v>
@@ -3366,7 +3366,7 @@
         <v>210</v>
       </c>
       <c r="G201" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H201" t="s">
         <v>9</v>
@@ -3377,7 +3377,7 @@
         <v>211</v>
       </c>
       <c r="G202" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H202" t="s">
         <v>9</v>
@@ -3388,7 +3388,7 @@
         <v>212</v>
       </c>
       <c r="G203" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H203" t="s">
         <v>9</v>
@@ -3399,7 +3399,7 @@
         <v>213</v>
       </c>
       <c r="G204" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H204" t="s">
         <v>9</v>
@@ -3410,7 +3410,7 @@
         <v>214</v>
       </c>
       <c r="G205" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H205" t="s">
         <v>9</v>
@@ -3421,7 +3421,7 @@
         <v>215</v>
       </c>
       <c r="G206" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H206" t="s">
         <v>9</v>
@@ -3432,7 +3432,7 @@
         <v>216</v>
       </c>
       <c r="G207" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H207" t="s">
         <v>9</v>
@@ -3443,7 +3443,7 @@
         <v>217</v>
       </c>
       <c r="G208" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H208" t="s">
         <v>9</v>
@@ -3454,7 +3454,7 @@
         <v>218</v>
       </c>
       <c r="G209" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H209" t="s">
         <v>9</v>
@@ -3465,7 +3465,7 @@
         <v>219</v>
       </c>
       <c r="G210" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H210" t="s">
         <v>9</v>
@@ -3476,7 +3476,7 @@
         <v>220</v>
       </c>
       <c r="G211" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H211" t="s">
         <v>9</v>
@@ -3487,7 +3487,7 @@
         <v>221</v>
       </c>
       <c r="G212" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H212" t="s">
         <v>9</v>
@@ -3498,7 +3498,7 @@
         <v>222</v>
       </c>
       <c r="G213" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H213" t="s">
         <v>9</v>
@@ -3509,7 +3509,7 @@
         <v>223</v>
       </c>
       <c r="G214" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H214" t="s">
         <v>9</v>
@@ -3520,7 +3520,7 @@
         <v>224</v>
       </c>
       <c r="G215" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H215" t="s">
         <v>9</v>
@@ -3531,7 +3531,7 @@
         <v>225</v>
       </c>
       <c r="G216" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H216" t="s">
         <v>9</v>
@@ -3542,7 +3542,7 @@
         <v>226</v>
       </c>
       <c r="G217" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H217" t="s">
         <v>9</v>
@@ -3553,7 +3553,7 @@
         <v>227</v>
       </c>
       <c r="G218" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H218" t="s">
         <v>9</v>
@@ -3564,7 +3564,7 @@
         <v>228</v>
       </c>
       <c r="G219" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H219" t="s">
         <v>9</v>
@@ -3575,7 +3575,7 @@
         <v>229</v>
       </c>
       <c r="G220" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H220" t="s">
         <v>9</v>
@@ -3586,7 +3586,7 @@
         <v>230</v>
       </c>
       <c r="G221" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H221" t="s">
         <v>9</v>
@@ -3597,7 +3597,7 @@
         <v>231</v>
       </c>
       <c r="G222" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H222" t="s">
         <v>9</v>
@@ -3608,7 +3608,7 @@
         <v>232</v>
       </c>
       <c r="G223" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H223" t="s">
         <v>9</v>
@@ -3619,7 +3619,7 @@
         <v>233</v>
       </c>
       <c r="G224" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H224" t="s">
         <v>9</v>
@@ -3630,7 +3630,7 @@
         <v>234</v>
       </c>
       <c r="G225" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H225" t="s">
         <v>9</v>
@@ -3641,7 +3641,7 @@
         <v>235</v>
       </c>
       <c r="G226" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H226" t="s">
         <v>9</v>
@@ -3652,7 +3652,7 @@
         <v>236</v>
       </c>
       <c r="G227" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H227" t="s">
         <v>9</v>
@@ -3663,7 +3663,7 @@
         <v>237</v>
       </c>
       <c r="G228" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H228" t="s">
         <v>9</v>
@@ -3674,7 +3674,7 @@
         <v>238</v>
       </c>
       <c r="G229" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H229" t="s">
         <v>9</v>
@@ -3685,7 +3685,7 @@
         <v>239</v>
       </c>
       <c r="G230" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H230" t="s">
         <v>9</v>
@@ -3696,7 +3696,7 @@
         <v>240</v>
       </c>
       <c r="G231" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H231" t="s">
         <v>9</v>
@@ -3707,7 +3707,7 @@
         <v>241</v>
       </c>
       <c r="G232" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H232" t="s">
         <v>9</v>
@@ -3718,7 +3718,7 @@
         <v>242</v>
       </c>
       <c r="G233" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H233" t="s">
         <v>9</v>
@@ -3729,7 +3729,7 @@
         <v>243</v>
       </c>
       <c r="G234" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H234" t="s">
         <v>9</v>
@@ -3740,7 +3740,7 @@
         <v>244</v>
       </c>
       <c r="G235" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H235" t="s">
         <v>9</v>
@@ -3751,7 +3751,7 @@
         <v>245</v>
       </c>
       <c r="G236" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H236" t="s">
         <v>9</v>
@@ -3762,7 +3762,7 @@
         <v>246</v>
       </c>
       <c r="G237" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H237" t="s">
         <v>9</v>
@@ -3773,7 +3773,7 @@
         <v>247</v>
       </c>
       <c r="G238" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H238" t="s">
         <v>9</v>
@@ -3784,7 +3784,7 @@
         <v>248</v>
       </c>
       <c r="G239" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H239" t="s">
         <v>9</v>
@@ -3795,7 +3795,7 @@
         <v>249</v>
       </c>
       <c r="G240" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H240" t="s">
         <v>9</v>
@@ -3806,7 +3806,7 @@
         <v>250</v>
       </c>
       <c r="G241" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H241" t="s">
         <v>9</v>
@@ -3817,7 +3817,7 @@
         <v>251</v>
       </c>
       <c r="G242" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H242" t="s">
         <v>9</v>
@@ -3828,7 +3828,7 @@
         <v>252</v>
       </c>
       <c r="G243" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H243" t="s">
         <v>9</v>
@@ -3839,7 +3839,7 @@
         <v>253</v>
       </c>
       <c r="G244" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H244" t="s">
         <v>9</v>
@@ -3850,7 +3850,7 @@
         <v>254</v>
       </c>
       <c r="G245" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H245" t="s">
         <v>9</v>
@@ -3861,7 +3861,7 @@
         <v>255</v>
       </c>
       <c r="G246" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H246" t="s">
         <v>9</v>
@@ -3872,7 +3872,7 @@
         <v>256</v>
       </c>
       <c r="G247" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H247" t="s">
         <v>9</v>
@@ -3883,7 +3883,7 @@
         <v>257</v>
       </c>
       <c r="G248" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H248" t="s">
         <v>9</v>
@@ -3894,7 +3894,7 @@
         <v>258</v>
       </c>
       <c r="G249" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H249" t="s">
         <v>9</v>
@@ -3905,7 +3905,7 @@
         <v>259</v>
       </c>
       <c r="G250" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H250" t="s">
         <v>9</v>
@@ -3916,7 +3916,7 @@
         <v>260</v>
       </c>
       <c r="G251" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H251" t="s">
         <v>9</v>
@@ -3927,7 +3927,7 @@
         <v>261</v>
       </c>
       <c r="G252" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H252" t="s">
         <v>9</v>
@@ -3938,7 +3938,7 @@
         <v>262</v>
       </c>
       <c r="G253" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H253" t="s">
         <v>9</v>
@@ -3949,7 +3949,7 @@
         <v>263</v>
       </c>
       <c r="G254" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H254" t="s">
         <v>9</v>
@@ -3960,7 +3960,7 @@
         <v>264</v>
       </c>
       <c r="G255" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H255" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
added comments and file information
</commit_message>
<xml_diff>
--- a/stationsinformation.xlsx
+++ b/stationsinformation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="264">
   <si>
     <t>Device</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t>ja</t>
-  </si>
-  <si>
-    <t>MZ Automation</t>
   </si>
   <si>
     <t>127.0.0.2</t>
@@ -1173,9 +1170,6 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
       <c r="G2" t="s">
         <v>10</v>
       </c>
@@ -1185,7 +1179,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
         <v>10</v>
@@ -1196,7 +1190,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
         <v>10</v>
@@ -1207,7 +1201,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
         <v>10</v>
@@ -1218,7 +1212,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
         <v>10</v>
@@ -1229,7 +1223,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G7" t="s">
         <v>10</v>
@@ -1240,7 +1234,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
         <v>10</v>
@@ -1251,7 +1245,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G9" t="s">
         <v>10</v>
@@ -1262,7 +1256,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G10" t="s">
         <v>10</v>
@@ -1273,7 +1267,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G11" t="s">
         <v>10</v>
@@ -1284,7 +1278,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" t="s">
         <v>10</v>
@@ -1295,7 +1289,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G13" t="s">
         <v>10</v>
@@ -1306,7 +1300,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" t="s">
         <v>10</v>
@@ -1317,7 +1311,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G15" t="s">
         <v>10</v>
@@ -1328,7 +1322,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
         <v>10</v>
@@ -1339,7 +1333,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G17" t="s">
         <v>10</v>
@@ -1350,7 +1344,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G18" t="s">
         <v>10</v>
@@ -1361,7 +1355,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G19" t="s">
         <v>10</v>
@@ -1372,7 +1366,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G20" t="s">
         <v>10</v>
@@ -1383,7 +1377,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G21" t="s">
         <v>10</v>
@@ -1394,7 +1388,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G22" t="s">
         <v>10</v>
@@ -1405,7 +1399,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G23" t="s">
         <v>10</v>
@@ -1416,7 +1410,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G24" t="s">
         <v>10</v>
@@ -1427,7 +1421,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G25" t="s">
         <v>10</v>
@@ -1438,7 +1432,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G26" t="s">
         <v>10</v>
@@ -1449,7 +1443,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G27" t="s">
         <v>10</v>
@@ -1460,7 +1454,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G28" t="s">
         <v>10</v>
@@ -1471,7 +1465,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G29" t="s">
         <v>10</v>
@@ -1482,7 +1476,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G30" t="s">
         <v>10</v>
@@ -1493,7 +1487,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G31" t="s">
         <v>10</v>
@@ -1504,7 +1498,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G32" t="s">
         <v>10</v>
@@ -1515,7 +1509,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G33" t="s">
         <v>10</v>
@@ -1526,7 +1520,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G34" t="s">
         <v>10</v>
@@ -1537,7 +1531,7 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G35" t="s">
         <v>10</v>
@@ -1548,7 +1542,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G36" t="s">
         <v>10</v>
@@ -1559,7 +1553,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G37" t="s">
         <v>10</v>
@@ -1570,7 +1564,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G38" t="s">
         <v>10</v>
@@ -1581,7 +1575,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G39" t="s">
         <v>10</v>
@@ -1592,7 +1586,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G40" t="s">
         <v>10</v>
@@ -1603,7 +1597,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G41" t="s">
         <v>10</v>
@@ -1614,7 +1608,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G42" t="s">
         <v>10</v>
@@ -1625,7 +1619,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G43" t="s">
         <v>10</v>
@@ -1636,7 +1630,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G44" t="s">
         <v>10</v>
@@ -1647,7 +1641,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G45" t="s">
         <v>10</v>
@@ -1658,7 +1652,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G46" t="s">
         <v>10</v>
@@ -1669,7 +1663,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G47" t="s">
         <v>10</v>
@@ -1680,7 +1674,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G48" t="s">
         <v>10</v>
@@ -1691,7 +1685,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G49" t="s">
         <v>10</v>
@@ -1702,7 +1696,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G50" t="s">
         <v>10</v>
@@ -1713,7 +1707,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G51" t="s">
         <v>10</v>
@@ -1724,7 +1718,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G52" t="s">
         <v>10</v>
@@ -1735,7 +1729,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G53" t="s">
         <v>10</v>
@@ -1746,7 +1740,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G54" t="s">
         <v>10</v>
@@ -1757,7 +1751,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G55" t="s">
         <v>10</v>
@@ -1768,7 +1762,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G56" t="s">
         <v>10</v>
@@ -1779,7 +1773,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G57" t="s">
         <v>10</v>
@@ -1790,7 +1784,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G58" t="s">
         <v>10</v>
@@ -1801,7 +1795,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G59" t="s">
         <v>10</v>
@@ -1812,7 +1806,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G60" t="s">
         <v>10</v>
@@ -1823,7 +1817,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G61" t="s">
         <v>10</v>
@@ -1834,7 +1828,7 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G62" t="s">
         <v>10</v>
@@ -1845,7 +1839,7 @@
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G63" t="s">
         <v>10</v>
@@ -1856,7 +1850,7 @@
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G64" t="s">
         <v>10</v>
@@ -1867,7 +1861,7 @@
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G65" t="s">
         <v>10</v>
@@ -1878,7 +1872,7 @@
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G66" t="s">
         <v>10</v>
@@ -1889,7 +1883,7 @@
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G67" t="s">
         <v>10</v>
@@ -1900,7 +1894,7 @@
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G68" t="s">
         <v>10</v>
@@ -1911,7 +1905,7 @@
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G69" t="s">
         <v>10</v>
@@ -1922,7 +1916,7 @@
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G70" t="s">
         <v>10</v>
@@ -1933,7 +1927,7 @@
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G71" t="s">
         <v>10</v>
@@ -1944,7 +1938,7 @@
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G72" t="s">
         <v>10</v>
@@ -1955,7 +1949,7 @@
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G73" t="s">
         <v>10</v>
@@ -1966,7 +1960,7 @@
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G74" t="s">
         <v>10</v>
@@ -1977,7 +1971,7 @@
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G75" t="s">
         <v>10</v>
@@ -1988,7 +1982,7 @@
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G76" t="s">
         <v>10</v>
@@ -1999,7 +1993,7 @@
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G77" t="s">
         <v>10</v>
@@ -2010,7 +2004,7 @@
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G78" t="s">
         <v>10</v>
@@ -2021,7 +2015,7 @@
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G79" t="s">
         <v>10</v>
@@ -2032,7 +2026,7 @@
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G80" t="s">
         <v>10</v>
@@ -2043,7 +2037,7 @@
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G81" t="s">
         <v>10</v>
@@ -2054,7 +2048,7 @@
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G82" t="s">
         <v>10</v>
@@ -2065,7 +2059,7 @@
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G83" t="s">
         <v>10</v>
@@ -2076,7 +2070,7 @@
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G84" t="s">
         <v>10</v>
@@ -2087,7 +2081,7 @@
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G85" t="s">
         <v>10</v>
@@ -2098,7 +2092,7 @@
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G86" t="s">
         <v>10</v>
@@ -2109,7 +2103,7 @@
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G87" t="s">
         <v>10</v>
@@ -2120,7 +2114,7 @@
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G88" t="s">
         <v>10</v>
@@ -2131,7 +2125,7 @@
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G89" t="s">
         <v>10</v>
@@ -2142,7 +2136,7 @@
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G90" t="s">
         <v>10</v>
@@ -2153,7 +2147,7 @@
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G91" t="s">
         <v>10</v>
@@ -2164,7 +2158,7 @@
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G92" t="s">
         <v>10</v>
@@ -2175,7 +2169,7 @@
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G93" t="s">
         <v>10</v>
@@ -2186,7 +2180,7 @@
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G94" t="s">
         <v>10</v>
@@ -2197,7 +2191,7 @@
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G95" t="s">
         <v>10</v>
@@ -2208,7 +2202,7 @@
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G96" t="s">
         <v>10</v>
@@ -2219,7 +2213,7 @@
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G97" t="s">
         <v>10</v>
@@ -2230,7 +2224,7 @@
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G98" t="s">
         <v>10</v>
@@ -2241,7 +2235,7 @@
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G99" t="s">
         <v>10</v>
@@ -2252,7 +2246,7 @@
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G100" t="s">
         <v>10</v>
@@ -2263,7 +2257,7 @@
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G101" t="s">
         <v>10</v>
@@ -2274,7 +2268,7 @@
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G102" t="s">
         <v>10</v>
@@ -2285,7 +2279,7 @@
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G103" t="s">
         <v>10</v>
@@ -2296,7 +2290,7 @@
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G104" t="s">
         <v>10</v>
@@ -2307,7 +2301,7 @@
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G105" t="s">
         <v>10</v>
@@ -2318,7 +2312,7 @@
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G106" t="s">
         <v>10</v>
@@ -2329,7 +2323,7 @@
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G107" t="s">
         <v>10</v>
@@ -2340,7 +2334,7 @@
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G108" t="s">
         <v>10</v>
@@ -2351,7 +2345,7 @@
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G109" t="s">
         <v>10</v>
@@ -2362,7 +2356,7 @@
     </row>
     <row r="110" spans="1:8">
       <c r="A110" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G110" t="s">
         <v>10</v>
@@ -2373,7 +2367,7 @@
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G111" t="s">
         <v>10</v>
@@ -2384,7 +2378,7 @@
     </row>
     <row r="112" spans="1:8">
       <c r="A112" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G112" t="s">
         <v>10</v>
@@ -2395,7 +2389,7 @@
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G113" t="s">
         <v>10</v>
@@ -2406,7 +2400,7 @@
     </row>
     <row r="114" spans="1:8">
       <c r="A114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G114" t="s">
         <v>10</v>
@@ -2417,7 +2411,7 @@
     </row>
     <row r="115" spans="1:8">
       <c r="A115" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G115" t="s">
         <v>10</v>
@@ -2428,7 +2422,7 @@
     </row>
     <row r="116" spans="1:8">
       <c r="A116" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G116" t="s">
         <v>10</v>
@@ -2439,7 +2433,7 @@
     </row>
     <row r="117" spans="1:8">
       <c r="A117" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G117" t="s">
         <v>10</v>
@@ -2450,7 +2444,7 @@
     </row>
     <row r="118" spans="1:8">
       <c r="A118" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G118" t="s">
         <v>10</v>
@@ -2461,7 +2455,7 @@
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G119" t="s">
         <v>10</v>
@@ -2472,7 +2466,7 @@
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G120" t="s">
         <v>10</v>
@@ -2483,7 +2477,7 @@
     </row>
     <row r="121" spans="1:8">
       <c r="A121" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G121" t="s">
         <v>10</v>
@@ -2494,7 +2488,7 @@
     </row>
     <row r="122" spans="1:8">
       <c r="A122" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G122" t="s">
         <v>10</v>
@@ -2505,7 +2499,7 @@
     </row>
     <row r="123" spans="1:8">
       <c r="A123" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G123" t="s">
         <v>10</v>
@@ -2516,7 +2510,7 @@
     </row>
     <row r="124" spans="1:8">
       <c r="A124" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G124" t="s">
         <v>10</v>
@@ -2527,7 +2521,7 @@
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G125" t="s">
         <v>10</v>
@@ -2538,7 +2532,7 @@
     </row>
     <row r="126" spans="1:8">
       <c r="A126" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G126" t="s">
         <v>10</v>
@@ -2549,7 +2543,7 @@
     </row>
     <row r="127" spans="1:8">
       <c r="A127" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G127" t="s">
         <v>10</v>
@@ -2560,7 +2554,7 @@
     </row>
     <row r="128" spans="1:8">
       <c r="A128" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G128" t="s">
         <v>10</v>
@@ -2571,7 +2565,7 @@
     </row>
     <row r="129" spans="1:8">
       <c r="A129" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G129" t="s">
         <v>10</v>
@@ -2582,7 +2576,7 @@
     </row>
     <row r="130" spans="1:8">
       <c r="A130" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G130" t="s">
         <v>10</v>
@@ -2593,7 +2587,7 @@
     </row>
     <row r="131" spans="1:8">
       <c r="A131" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G131" t="s">
         <v>10</v>
@@ -2604,7 +2598,7 @@
     </row>
     <row r="132" spans="1:8">
       <c r="A132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G132" t="s">
         <v>10</v>
@@ -2615,7 +2609,7 @@
     </row>
     <row r="133" spans="1:8">
       <c r="A133" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G133" t="s">
         <v>10</v>
@@ -2626,7 +2620,7 @@
     </row>
     <row r="134" spans="1:8">
       <c r="A134" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G134" t="s">
         <v>10</v>
@@ -2637,7 +2631,7 @@
     </row>
     <row r="135" spans="1:8">
       <c r="A135" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G135" t="s">
         <v>10</v>
@@ -2648,7 +2642,7 @@
     </row>
     <row r="136" spans="1:8">
       <c r="A136" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G136" t="s">
         <v>10</v>
@@ -2659,7 +2653,7 @@
     </row>
     <row r="137" spans="1:8">
       <c r="A137" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G137" t="s">
         <v>10</v>
@@ -2670,7 +2664,7 @@
     </row>
     <row r="138" spans="1:8">
       <c r="A138" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G138" t="s">
         <v>10</v>
@@ -2681,7 +2675,7 @@
     </row>
     <row r="139" spans="1:8">
       <c r="A139" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G139" t="s">
         <v>10</v>
@@ -2692,7 +2686,7 @@
     </row>
     <row r="140" spans="1:8">
       <c r="A140" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G140" t="s">
         <v>10</v>
@@ -2703,7 +2697,7 @@
     </row>
     <row r="141" spans="1:8">
       <c r="A141" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G141" t="s">
         <v>10</v>
@@ -2714,7 +2708,7 @@
     </row>
     <row r="142" spans="1:8">
       <c r="A142" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G142" t="s">
         <v>10</v>
@@ -2725,7 +2719,7 @@
     </row>
     <row r="143" spans="1:8">
       <c r="A143" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G143" t="s">
         <v>10</v>
@@ -2736,7 +2730,7 @@
     </row>
     <row r="144" spans="1:8">
       <c r="A144" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G144" t="s">
         <v>10</v>
@@ -2747,7 +2741,7 @@
     </row>
     <row r="145" spans="1:8">
       <c r="A145" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G145" t="s">
         <v>10</v>
@@ -2758,7 +2752,7 @@
     </row>
     <row r="146" spans="1:8">
       <c r="A146" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G146" t="s">
         <v>10</v>
@@ -2769,7 +2763,7 @@
     </row>
     <row r="147" spans="1:8">
       <c r="A147" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G147" t="s">
         <v>10</v>
@@ -2780,7 +2774,7 @@
     </row>
     <row r="148" spans="1:8">
       <c r="A148" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G148" t="s">
         <v>10</v>
@@ -2791,7 +2785,7 @@
     </row>
     <row r="149" spans="1:8">
       <c r="A149" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G149" t="s">
         <v>10</v>
@@ -2802,7 +2796,7 @@
     </row>
     <row r="150" spans="1:8">
       <c r="A150" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G150" t="s">
         <v>10</v>
@@ -2813,7 +2807,7 @@
     </row>
     <row r="151" spans="1:8">
       <c r="A151" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G151" t="s">
         <v>10</v>
@@ -2824,7 +2818,7 @@
     </row>
     <row r="152" spans="1:8">
       <c r="A152" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G152" t="s">
         <v>10</v>
@@ -2835,7 +2829,7 @@
     </row>
     <row r="153" spans="1:8">
       <c r="A153" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G153" t="s">
         <v>10</v>
@@ -2846,7 +2840,7 @@
     </row>
     <row r="154" spans="1:8">
       <c r="A154" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G154" t="s">
         <v>10</v>
@@ -2857,7 +2851,7 @@
     </row>
     <row r="155" spans="1:8">
       <c r="A155" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G155" t="s">
         <v>10</v>
@@ -2868,7 +2862,7 @@
     </row>
     <row r="156" spans="1:8">
       <c r="A156" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G156" t="s">
         <v>10</v>
@@ -2879,7 +2873,7 @@
     </row>
     <row r="157" spans="1:8">
       <c r="A157" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G157" t="s">
         <v>10</v>
@@ -2890,7 +2884,7 @@
     </row>
     <row r="158" spans="1:8">
       <c r="A158" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G158" t="s">
         <v>10</v>
@@ -2901,7 +2895,7 @@
     </row>
     <row r="159" spans="1:8">
       <c r="A159" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G159" t="s">
         <v>10</v>
@@ -2912,7 +2906,7 @@
     </row>
     <row r="160" spans="1:8">
       <c r="A160" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G160" t="s">
         <v>10</v>
@@ -2923,7 +2917,7 @@
     </row>
     <row r="161" spans="1:8">
       <c r="A161" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G161" t="s">
         <v>10</v>
@@ -2934,7 +2928,7 @@
     </row>
     <row r="162" spans="1:8">
       <c r="A162" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G162" t="s">
         <v>10</v>
@@ -2945,7 +2939,7 @@
     </row>
     <row r="163" spans="1:8">
       <c r="A163" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G163" t="s">
         <v>10</v>
@@ -2956,7 +2950,7 @@
     </row>
     <row r="164" spans="1:8">
       <c r="A164" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G164" t="s">
         <v>10</v>
@@ -2967,7 +2961,7 @@
     </row>
     <row r="165" spans="1:8">
       <c r="A165" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G165" t="s">
         <v>10</v>
@@ -2978,7 +2972,7 @@
     </row>
     <row r="166" spans="1:8">
       <c r="A166" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G166" t="s">
         <v>10</v>
@@ -2989,7 +2983,7 @@
     </row>
     <row r="167" spans="1:8">
       <c r="A167" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G167" t="s">
         <v>10</v>
@@ -3000,7 +2994,7 @@
     </row>
     <row r="168" spans="1:8">
       <c r="A168" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G168" t="s">
         <v>10</v>
@@ -3011,7 +3005,7 @@
     </row>
     <row r="169" spans="1:8">
       <c r="A169" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G169" t="s">
         <v>10</v>
@@ -3022,7 +3016,7 @@
     </row>
     <row r="170" spans="1:8">
       <c r="A170" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G170" t="s">
         <v>10</v>
@@ -3033,7 +3027,7 @@
     </row>
     <row r="171" spans="1:8">
       <c r="A171" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G171" t="s">
         <v>10</v>
@@ -3044,7 +3038,7 @@
     </row>
     <row r="172" spans="1:8">
       <c r="A172" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G172" t="s">
         <v>10</v>
@@ -3055,7 +3049,7 @@
     </row>
     <row r="173" spans="1:8">
       <c r="A173" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G173" t="s">
         <v>10</v>
@@ -3066,7 +3060,7 @@
     </row>
     <row r="174" spans="1:8">
       <c r="A174" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G174" t="s">
         <v>10</v>
@@ -3077,7 +3071,7 @@
     </row>
     <row r="175" spans="1:8">
       <c r="A175" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G175" t="s">
         <v>10</v>
@@ -3088,7 +3082,7 @@
     </row>
     <row r="176" spans="1:8">
       <c r="A176" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G176" t="s">
         <v>10</v>
@@ -3099,7 +3093,7 @@
     </row>
     <row r="177" spans="1:8">
       <c r="A177" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G177" t="s">
         <v>10</v>
@@ -3110,7 +3104,7 @@
     </row>
     <row r="178" spans="1:8">
       <c r="A178" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G178" t="s">
         <v>10</v>
@@ -3121,7 +3115,7 @@
     </row>
     <row r="179" spans="1:8">
       <c r="A179" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G179" t="s">
         <v>10</v>
@@ -3132,7 +3126,7 @@
     </row>
     <row r="180" spans="1:8">
       <c r="A180" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G180" t="s">
         <v>10</v>
@@ -3143,7 +3137,7 @@
     </row>
     <row r="181" spans="1:8">
       <c r="A181" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G181" t="s">
         <v>10</v>
@@ -3154,7 +3148,7 @@
     </row>
     <row r="182" spans="1:8">
       <c r="A182" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G182" t="s">
         <v>10</v>
@@ -3165,7 +3159,7 @@
     </row>
     <row r="183" spans="1:8">
       <c r="A183" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G183" t="s">
         <v>10</v>
@@ -3176,7 +3170,7 @@
     </row>
     <row r="184" spans="1:8">
       <c r="A184" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G184" t="s">
         <v>10</v>
@@ -3187,7 +3181,7 @@
     </row>
     <row r="185" spans="1:8">
       <c r="A185" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G185" t="s">
         <v>10</v>
@@ -3198,7 +3192,7 @@
     </row>
     <row r="186" spans="1:8">
       <c r="A186" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G186" t="s">
         <v>10</v>
@@ -3209,7 +3203,7 @@
     </row>
     <row r="187" spans="1:8">
       <c r="A187" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G187" t="s">
         <v>10</v>
@@ -3220,7 +3214,7 @@
     </row>
     <row r="188" spans="1:8">
       <c r="A188" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G188" t="s">
         <v>10</v>
@@ -3231,7 +3225,7 @@
     </row>
     <row r="189" spans="1:8">
       <c r="A189" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G189" t="s">
         <v>10</v>
@@ -3242,7 +3236,7 @@
     </row>
     <row r="190" spans="1:8">
       <c r="A190" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G190" t="s">
         <v>10</v>
@@ -3253,7 +3247,7 @@
     </row>
     <row r="191" spans="1:8">
       <c r="A191" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G191" t="s">
         <v>10</v>
@@ -3264,7 +3258,7 @@
     </row>
     <row r="192" spans="1:8">
       <c r="A192" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G192" t="s">
         <v>10</v>
@@ -3275,7 +3269,7 @@
     </row>
     <row r="193" spans="1:8">
       <c r="A193" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G193" t="s">
         <v>10</v>
@@ -3286,7 +3280,7 @@
     </row>
     <row r="194" spans="1:8">
       <c r="A194" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G194" t="s">
         <v>10</v>
@@ -3297,7 +3291,7 @@
     </row>
     <row r="195" spans="1:8">
       <c r="A195" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G195" t="s">
         <v>10</v>
@@ -3308,7 +3302,7 @@
     </row>
     <row r="196" spans="1:8">
       <c r="A196" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G196" t="s">
         <v>10</v>
@@ -3319,7 +3313,7 @@
     </row>
     <row r="197" spans="1:8">
       <c r="A197" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G197" t="s">
         <v>10</v>
@@ -3330,7 +3324,7 @@
     </row>
     <row r="198" spans="1:8">
       <c r="A198" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G198" t="s">
         <v>10</v>
@@ -3341,7 +3335,7 @@
     </row>
     <row r="199" spans="1:8">
       <c r="A199" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G199" t="s">
         <v>10</v>
@@ -3352,7 +3346,7 @@
     </row>
     <row r="200" spans="1:8">
       <c r="A200" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G200" t="s">
         <v>10</v>
@@ -3363,7 +3357,7 @@
     </row>
     <row r="201" spans="1:8">
       <c r="A201" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G201" t="s">
         <v>10</v>
@@ -3374,7 +3368,7 @@
     </row>
     <row r="202" spans="1:8">
       <c r="A202" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G202" t="s">
         <v>10</v>
@@ -3385,7 +3379,7 @@
     </row>
     <row r="203" spans="1:8">
       <c r="A203" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G203" t="s">
         <v>10</v>
@@ -3396,7 +3390,7 @@
     </row>
     <row r="204" spans="1:8">
       <c r="A204" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G204" t="s">
         <v>10</v>
@@ -3407,7 +3401,7 @@
     </row>
     <row r="205" spans="1:8">
       <c r="A205" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G205" t="s">
         <v>10</v>
@@ -3418,7 +3412,7 @@
     </row>
     <row r="206" spans="1:8">
       <c r="A206" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G206" t="s">
         <v>10</v>
@@ -3429,7 +3423,7 @@
     </row>
     <row r="207" spans="1:8">
       <c r="A207" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G207" t="s">
         <v>10</v>
@@ -3440,7 +3434,7 @@
     </row>
     <row r="208" spans="1:8">
       <c r="A208" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G208" t="s">
         <v>10</v>
@@ -3451,7 +3445,7 @@
     </row>
     <row r="209" spans="1:8">
       <c r="A209" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G209" t="s">
         <v>10</v>
@@ -3462,7 +3456,7 @@
     </row>
     <row r="210" spans="1:8">
       <c r="A210" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G210" t="s">
         <v>10</v>
@@ -3473,7 +3467,7 @@
     </row>
     <row r="211" spans="1:8">
       <c r="A211" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G211" t="s">
         <v>10</v>
@@ -3484,7 +3478,7 @@
     </row>
     <row r="212" spans="1:8">
       <c r="A212" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G212" t="s">
         <v>10</v>
@@ -3495,7 +3489,7 @@
     </row>
     <row r="213" spans="1:8">
       <c r="A213" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G213" t="s">
         <v>10</v>
@@ -3506,7 +3500,7 @@
     </row>
     <row r="214" spans="1:8">
       <c r="A214" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G214" t="s">
         <v>10</v>
@@ -3517,7 +3511,7 @@
     </row>
     <row r="215" spans="1:8">
       <c r="A215" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G215" t="s">
         <v>10</v>
@@ -3528,7 +3522,7 @@
     </row>
     <row r="216" spans="1:8">
       <c r="A216" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G216" t="s">
         <v>10</v>
@@ -3539,7 +3533,7 @@
     </row>
     <row r="217" spans="1:8">
       <c r="A217" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G217" t="s">
         <v>10</v>
@@ -3550,7 +3544,7 @@
     </row>
     <row r="218" spans="1:8">
       <c r="A218" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G218" t="s">
         <v>10</v>
@@ -3561,7 +3555,7 @@
     </row>
     <row r="219" spans="1:8">
       <c r="A219" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G219" t="s">
         <v>10</v>
@@ -3572,7 +3566,7 @@
     </row>
     <row r="220" spans="1:8">
       <c r="A220" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G220" t="s">
         <v>10</v>
@@ -3583,7 +3577,7 @@
     </row>
     <row r="221" spans="1:8">
       <c r="A221" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G221" t="s">
         <v>10</v>
@@ -3594,7 +3588,7 @@
     </row>
     <row r="222" spans="1:8">
       <c r="A222" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G222" t="s">
         <v>10</v>
@@ -3605,7 +3599,7 @@
     </row>
     <row r="223" spans="1:8">
       <c r="A223" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G223" t="s">
         <v>10</v>
@@ -3616,7 +3610,7 @@
     </row>
     <row r="224" spans="1:8">
       <c r="A224" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G224" t="s">
         <v>10</v>
@@ -3627,7 +3621,7 @@
     </row>
     <row r="225" spans="1:8">
       <c r="A225" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G225" t="s">
         <v>10</v>
@@ -3638,7 +3632,7 @@
     </row>
     <row r="226" spans="1:8">
       <c r="A226" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G226" t="s">
         <v>10</v>
@@ -3649,7 +3643,7 @@
     </row>
     <row r="227" spans="1:8">
       <c r="A227" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G227" t="s">
         <v>10</v>
@@ -3660,7 +3654,7 @@
     </row>
     <row r="228" spans="1:8">
       <c r="A228" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G228" t="s">
         <v>10</v>
@@ -3671,7 +3665,7 @@
     </row>
     <row r="229" spans="1:8">
       <c r="A229" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G229" t="s">
         <v>10</v>
@@ -3682,7 +3676,7 @@
     </row>
     <row r="230" spans="1:8">
       <c r="A230" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G230" t="s">
         <v>10</v>
@@ -3693,7 +3687,7 @@
     </row>
     <row r="231" spans="1:8">
       <c r="A231" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G231" t="s">
         <v>10</v>
@@ -3704,7 +3698,7 @@
     </row>
     <row r="232" spans="1:8">
       <c r="A232" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G232" t="s">
         <v>10</v>
@@ -3715,7 +3709,7 @@
     </row>
     <row r="233" spans="1:8">
       <c r="A233" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G233" t="s">
         <v>10</v>
@@ -3726,7 +3720,7 @@
     </row>
     <row r="234" spans="1:8">
       <c r="A234" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G234" t="s">
         <v>10</v>
@@ -3737,7 +3731,7 @@
     </row>
     <row r="235" spans="1:8">
       <c r="A235" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G235" t="s">
         <v>10</v>
@@ -3748,7 +3742,7 @@
     </row>
     <row r="236" spans="1:8">
       <c r="A236" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G236" t="s">
         <v>10</v>
@@ -3759,7 +3753,7 @@
     </row>
     <row r="237" spans="1:8">
       <c r="A237" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G237" t="s">
         <v>10</v>
@@ -3770,7 +3764,7 @@
     </row>
     <row r="238" spans="1:8">
       <c r="A238" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G238" t="s">
         <v>10</v>
@@ -3781,7 +3775,7 @@
     </row>
     <row r="239" spans="1:8">
       <c r="A239" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G239" t="s">
         <v>10</v>
@@ -3792,7 +3786,7 @@
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G240" t="s">
         <v>10</v>
@@ -3803,7 +3797,7 @@
     </row>
     <row r="241" spans="1:8">
       <c r="A241" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G241" t="s">
         <v>10</v>
@@ -3814,7 +3808,7 @@
     </row>
     <row r="242" spans="1:8">
       <c r="A242" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G242" t="s">
         <v>10</v>
@@ -3825,7 +3819,7 @@
     </row>
     <row r="243" spans="1:8">
       <c r="A243" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G243" t="s">
         <v>10</v>
@@ -3836,7 +3830,7 @@
     </row>
     <row r="244" spans="1:8">
       <c r="A244" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G244" t="s">
         <v>10</v>
@@ -3847,7 +3841,7 @@
     </row>
     <row r="245" spans="1:8">
       <c r="A245" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G245" t="s">
         <v>10</v>
@@ -3858,7 +3852,7 @@
     </row>
     <row r="246" spans="1:8">
       <c r="A246" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G246" t="s">
         <v>10</v>
@@ -3869,7 +3863,7 @@
     </row>
     <row r="247" spans="1:8">
       <c r="A247" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G247" t="s">
         <v>10</v>
@@ -3880,7 +3874,7 @@
     </row>
     <row r="248" spans="1:8">
       <c r="A248" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G248" t="s">
         <v>10</v>
@@ -3891,7 +3885,7 @@
     </row>
     <row r="249" spans="1:8">
       <c r="A249" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G249" t="s">
         <v>10</v>
@@ -3902,7 +3896,7 @@
     </row>
     <row r="250" spans="1:8">
       <c r="A250" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G250" t="s">
         <v>10</v>
@@ -3913,7 +3907,7 @@
     </row>
     <row r="251" spans="1:8">
       <c r="A251" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G251" t="s">
         <v>10</v>
@@ -3924,7 +3918,7 @@
     </row>
     <row r="252" spans="1:8">
       <c r="A252" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G252" t="s">
         <v>10</v>
@@ -3935,7 +3929,7 @@
     </row>
     <row r="253" spans="1:8">
       <c r="A253" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G253" t="s">
         <v>10</v>
@@ -3946,7 +3940,7 @@
     </row>
     <row r="254" spans="1:8">
       <c r="A254" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G254" t="s">
         <v>10</v>
@@ -3957,7 +3951,7 @@
     </row>
     <row r="255" spans="1:8">
       <c r="A255" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G255" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
closing connection after each connect, now MMS works for all IEDs
</commit_message>
<xml_diff>
--- a/stationsinformation.xlsx
+++ b/stationsinformation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="264">
   <si>
     <t>Device</t>
   </si>
@@ -1184,2772 +1184,3528 @@
       <c r="A3" t="s">
         <v>12</v>
       </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
       <c r="G3" t="s">
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>13</v>
       </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
       <c r="G4" t="s">
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>14</v>
       </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
       <c r="G5" t="s">
         <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>15</v>
       </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
       <c r="G6" t="s">
         <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>16</v>
       </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
       <c r="G7" t="s">
         <v>10</v>
       </c>
       <c r="H7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>17</v>
       </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
       <c r="G8" t="s">
         <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>18</v>
       </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
       <c r="G9" t="s">
         <v>10</v>
       </c>
       <c r="H9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>19</v>
       </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
       <c r="G10" t="s">
         <v>10</v>
       </c>
       <c r="H10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>20</v>
       </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
       <c r="G11" t="s">
         <v>10</v>
       </c>
       <c r="H11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>21</v>
       </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
       <c r="G12" t="s">
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>22</v>
       </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
       <c r="G13" t="s">
         <v>10</v>
       </c>
       <c r="H13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>23</v>
       </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
       <c r="G14" t="s">
         <v>10</v>
       </c>
       <c r="H14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>24</v>
       </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
       <c r="G15" t="s">
         <v>10</v>
       </c>
       <c r="H15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>25</v>
       </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
       <c r="G16" t="s">
         <v>10</v>
       </c>
       <c r="H16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>26</v>
       </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
       <c r="G17" t="s">
         <v>10</v>
       </c>
       <c r="H17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>27</v>
       </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
       <c r="G18" t="s">
         <v>10</v>
       </c>
       <c r="H18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>28</v>
       </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
       <c r="G19" t="s">
         <v>10</v>
       </c>
       <c r="H19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>29</v>
       </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
       <c r="G20" t="s">
         <v>10</v>
       </c>
       <c r="H20" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>30</v>
       </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
       <c r="G21" t="s">
         <v>10</v>
       </c>
       <c r="H21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
         <v>31</v>
       </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
       <c r="G22" t="s">
         <v>10</v>
       </c>
       <c r="H22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
         <v>32</v>
       </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
       <c r="G23" t="s">
         <v>10</v>
       </c>
       <c r="H23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
         <v>33</v>
       </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
       <c r="G24" t="s">
         <v>10</v>
       </c>
       <c r="H24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
         <v>34</v>
       </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
       <c r="G25" t="s">
         <v>10</v>
       </c>
       <c r="H25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
         <v>35</v>
       </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
       <c r="G26" t="s">
         <v>10</v>
       </c>
       <c r="H26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
         <v>36</v>
       </c>
+      <c r="C27" t="s">
+        <v>11</v>
+      </c>
       <c r="G27" t="s">
         <v>10</v>
       </c>
       <c r="H27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
         <v>37</v>
       </c>
+      <c r="C28" t="s">
+        <v>11</v>
+      </c>
       <c r="G28" t="s">
         <v>10</v>
       </c>
       <c r="H28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
         <v>38</v>
       </c>
+      <c r="C29" t="s">
+        <v>11</v>
+      </c>
       <c r="G29" t="s">
         <v>10</v>
       </c>
       <c r="H29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
         <v>39</v>
       </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
       <c r="G30" t="s">
         <v>10</v>
       </c>
       <c r="H30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
         <v>40</v>
       </c>
+      <c r="C31" t="s">
+        <v>11</v>
+      </c>
       <c r="G31" t="s">
         <v>10</v>
       </c>
       <c r="H31" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
         <v>41</v>
       </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
       <c r="G32" t="s">
         <v>10</v>
       </c>
       <c r="H32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>42</v>
       </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
       <c r="G33" t="s">
         <v>10</v>
       </c>
       <c r="H33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>43</v>
       </c>
+      <c r="C34" t="s">
+        <v>11</v>
+      </c>
       <c r="G34" t="s">
         <v>10</v>
       </c>
       <c r="H34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>44</v>
       </c>
+      <c r="C35" t="s">
+        <v>11</v>
+      </c>
       <c r="G35" t="s">
         <v>10</v>
       </c>
       <c r="H35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
         <v>45</v>
       </c>
+      <c r="C36" t="s">
+        <v>11</v>
+      </c>
       <c r="G36" t="s">
         <v>10</v>
       </c>
       <c r="H36" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
         <v>46</v>
       </c>
+      <c r="C37" t="s">
+        <v>11</v>
+      </c>
       <c r="G37" t="s">
         <v>10</v>
       </c>
       <c r="H37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>47</v>
       </c>
+      <c r="C38" t="s">
+        <v>11</v>
+      </c>
       <c r="G38" t="s">
         <v>10</v>
       </c>
       <c r="H38" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>48</v>
       </c>
+      <c r="C39" t="s">
+        <v>11</v>
+      </c>
       <c r="G39" t="s">
         <v>10</v>
       </c>
       <c r="H39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>49</v>
       </c>
+      <c r="C40" t="s">
+        <v>11</v>
+      </c>
       <c r="G40" t="s">
         <v>10</v>
       </c>
       <c r="H40" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
         <v>50</v>
       </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
       <c r="G41" t="s">
         <v>10</v>
       </c>
       <c r="H41" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>51</v>
       </c>
+      <c r="C42" t="s">
+        <v>11</v>
+      </c>
       <c r="G42" t="s">
         <v>10</v>
       </c>
       <c r="H42" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
         <v>52</v>
       </c>
+      <c r="C43" t="s">
+        <v>11</v>
+      </c>
       <c r="G43" t="s">
         <v>10</v>
       </c>
       <c r="H43" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
         <v>53</v>
       </c>
+      <c r="C44" t="s">
+        <v>11</v>
+      </c>
       <c r="G44" t="s">
         <v>10</v>
       </c>
       <c r="H44" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
         <v>54</v>
       </c>
+      <c r="C45" t="s">
+        <v>11</v>
+      </c>
       <c r="G45" t="s">
         <v>10</v>
       </c>
       <c r="H45" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
         <v>55</v>
       </c>
+      <c r="C46" t="s">
+        <v>11</v>
+      </c>
       <c r="G46" t="s">
         <v>10</v>
       </c>
       <c r="H46" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
         <v>56</v>
       </c>
+      <c r="C47" t="s">
+        <v>11</v>
+      </c>
       <c r="G47" t="s">
         <v>10</v>
       </c>
       <c r="H47" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>57</v>
       </c>
+      <c r="C48" t="s">
+        <v>11</v>
+      </c>
       <c r="G48" t="s">
         <v>10</v>
       </c>
       <c r="H48" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>58</v>
       </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
       <c r="G49" t="s">
         <v>10</v>
       </c>
       <c r="H49" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
         <v>59</v>
       </c>
+      <c r="C50" t="s">
+        <v>11</v>
+      </c>
       <c r="G50" t="s">
         <v>10</v>
       </c>
       <c r="H50" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
         <v>60</v>
       </c>
+      <c r="C51" t="s">
+        <v>11</v>
+      </c>
       <c r="G51" t="s">
         <v>10</v>
       </c>
       <c r="H51" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
         <v>61</v>
       </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
       <c r="G52" t="s">
         <v>10</v>
       </c>
       <c r="H52" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
         <v>62</v>
       </c>
+      <c r="C53" t="s">
+        <v>11</v>
+      </c>
       <c r="G53" t="s">
         <v>10</v>
       </c>
       <c r="H53" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
         <v>63</v>
       </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
       <c r="G54" t="s">
         <v>10</v>
       </c>
       <c r="H54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
         <v>64</v>
       </c>
+      <c r="C55" t="s">
+        <v>11</v>
+      </c>
       <c r="G55" t="s">
         <v>10</v>
       </c>
       <c r="H55" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
         <v>65</v>
       </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
       <c r="G56" t="s">
         <v>10</v>
       </c>
       <c r="H56" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
         <v>66</v>
       </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
       <c r="G57" t="s">
         <v>10</v>
       </c>
       <c r="H57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
         <v>67</v>
       </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
       <c r="G58" t="s">
         <v>10</v>
       </c>
       <c r="H58" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
         <v>68</v>
       </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
       <c r="G59" t="s">
         <v>10</v>
       </c>
       <c r="H59" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
         <v>69</v>
       </c>
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
       <c r="G60" t="s">
         <v>10</v>
       </c>
       <c r="H60" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
         <v>70</v>
       </c>
+      <c r="C61" t="s">
+        <v>11</v>
+      </c>
       <c r="G61" t="s">
         <v>10</v>
       </c>
       <c r="H61" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
         <v>71</v>
       </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
       <c r="G62" t="s">
         <v>10</v>
       </c>
       <c r="H62" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
         <v>72</v>
       </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
       <c r="G63" t="s">
         <v>10</v>
       </c>
       <c r="H63" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
         <v>73</v>
       </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
       <c r="G64" t="s">
         <v>10</v>
       </c>
       <c r="H64" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
         <v>74</v>
       </c>
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
       <c r="G65" t="s">
         <v>10</v>
       </c>
       <c r="H65" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
         <v>75</v>
       </c>
+      <c r="C66" t="s">
+        <v>11</v>
+      </c>
       <c r="G66" t="s">
         <v>10</v>
       </c>
       <c r="H66" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
         <v>76</v>
       </c>
+      <c r="C67" t="s">
+        <v>11</v>
+      </c>
       <c r="G67" t="s">
         <v>10</v>
       </c>
       <c r="H67" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
         <v>77</v>
       </c>
+      <c r="C68" t="s">
+        <v>11</v>
+      </c>
       <c r="G68" t="s">
         <v>10</v>
       </c>
       <c r="H68" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
         <v>78</v>
       </c>
+      <c r="C69" t="s">
+        <v>11</v>
+      </c>
       <c r="G69" t="s">
         <v>10</v>
       </c>
       <c r="H69" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
         <v>79</v>
       </c>
+      <c r="C70" t="s">
+        <v>11</v>
+      </c>
       <c r="G70" t="s">
         <v>10</v>
       </c>
       <c r="H70" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
         <v>80</v>
       </c>
+      <c r="C71" t="s">
+        <v>11</v>
+      </c>
       <c r="G71" t="s">
         <v>10</v>
       </c>
       <c r="H71" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
         <v>81</v>
       </c>
+      <c r="C72" t="s">
+        <v>11</v>
+      </c>
       <c r="G72" t="s">
         <v>10</v>
       </c>
       <c r="H72" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
         <v>82</v>
       </c>
+      <c r="C73" t="s">
+        <v>11</v>
+      </c>
       <c r="G73" t="s">
         <v>10</v>
       </c>
       <c r="H73" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
         <v>83</v>
       </c>
+      <c r="C74" t="s">
+        <v>11</v>
+      </c>
       <c r="G74" t="s">
         <v>10</v>
       </c>
       <c r="H74" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
         <v>84</v>
       </c>
+      <c r="C75" t="s">
+        <v>11</v>
+      </c>
       <c r="G75" t="s">
         <v>10</v>
       </c>
       <c r="H75" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
         <v>85</v>
       </c>
+      <c r="C76" t="s">
+        <v>11</v>
+      </c>
       <c r="G76" t="s">
         <v>10</v>
       </c>
       <c r="H76" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
         <v>86</v>
       </c>
+      <c r="C77" t="s">
+        <v>11</v>
+      </c>
       <c r="G77" t="s">
         <v>10</v>
       </c>
       <c r="H77" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
         <v>87</v>
       </c>
+      <c r="C78" t="s">
+        <v>11</v>
+      </c>
       <c r="G78" t="s">
         <v>10</v>
       </c>
       <c r="H78" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
         <v>88</v>
       </c>
+      <c r="C79" t="s">
+        <v>11</v>
+      </c>
       <c r="G79" t="s">
         <v>10</v>
       </c>
       <c r="H79" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
         <v>89</v>
       </c>
+      <c r="C80" t="s">
+        <v>11</v>
+      </c>
       <c r="G80" t="s">
         <v>10</v>
       </c>
       <c r="H80" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
         <v>90</v>
       </c>
+      <c r="C81" t="s">
+        <v>11</v>
+      </c>
       <c r="G81" t="s">
         <v>10</v>
       </c>
       <c r="H81" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
         <v>91</v>
       </c>
+      <c r="C82" t="s">
+        <v>11</v>
+      </c>
       <c r="G82" t="s">
         <v>10</v>
       </c>
       <c r="H82" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
         <v>92</v>
       </c>
+      <c r="C83" t="s">
+        <v>11</v>
+      </c>
       <c r="G83" t="s">
         <v>10</v>
       </c>
       <c r="H83" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
         <v>93</v>
       </c>
+      <c r="C84" t="s">
+        <v>11</v>
+      </c>
       <c r="G84" t="s">
         <v>10</v>
       </c>
       <c r="H84" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
         <v>94</v>
       </c>
+      <c r="C85" t="s">
+        <v>11</v>
+      </c>
       <c r="G85" t="s">
         <v>10</v>
       </c>
       <c r="H85" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
         <v>95</v>
       </c>
+      <c r="C86" t="s">
+        <v>11</v>
+      </c>
       <c r="G86" t="s">
         <v>10</v>
       </c>
       <c r="H86" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
         <v>96</v>
       </c>
+      <c r="C87" t="s">
+        <v>11</v>
+      </c>
       <c r="G87" t="s">
         <v>10</v>
       </c>
       <c r="H87" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
         <v>97</v>
       </c>
+      <c r="C88" t="s">
+        <v>11</v>
+      </c>
       <c r="G88" t="s">
         <v>10</v>
       </c>
       <c r="H88" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
         <v>98</v>
       </c>
+      <c r="C89" t="s">
+        <v>11</v>
+      </c>
       <c r="G89" t="s">
         <v>10</v>
       </c>
       <c r="H89" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
         <v>99</v>
       </c>
+      <c r="C90" t="s">
+        <v>11</v>
+      </c>
       <c r="G90" t="s">
         <v>10</v>
       </c>
       <c r="H90" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
         <v>100</v>
       </c>
+      <c r="C91" t="s">
+        <v>11</v>
+      </c>
       <c r="G91" t="s">
         <v>10</v>
       </c>
       <c r="H91" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
         <v>101</v>
       </c>
+      <c r="C92" t="s">
+        <v>11</v>
+      </c>
       <c r="G92" t="s">
         <v>10</v>
       </c>
       <c r="H92" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
         <v>102</v>
       </c>
+      <c r="C93" t="s">
+        <v>11</v>
+      </c>
       <c r="G93" t="s">
         <v>10</v>
       </c>
       <c r="H93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
         <v>103</v>
       </c>
+      <c r="C94" t="s">
+        <v>11</v>
+      </c>
       <c r="G94" t="s">
         <v>10</v>
       </c>
       <c r="H94" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
         <v>104</v>
       </c>
+      <c r="C95" t="s">
+        <v>11</v>
+      </c>
       <c r="G95" t="s">
         <v>10</v>
       </c>
       <c r="H95" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
         <v>105</v>
       </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
       <c r="G96" t="s">
         <v>10</v>
       </c>
       <c r="H96" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
         <v>106</v>
       </c>
+      <c r="C97" t="s">
+        <v>11</v>
+      </c>
       <c r="G97" t="s">
         <v>10</v>
       </c>
       <c r="H97" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
         <v>107</v>
       </c>
+      <c r="C98" t="s">
+        <v>11</v>
+      </c>
       <c r="G98" t="s">
         <v>10</v>
       </c>
       <c r="H98" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
         <v>108</v>
       </c>
+      <c r="C99" t="s">
+        <v>11</v>
+      </c>
       <c r="G99" t="s">
         <v>10</v>
       </c>
       <c r="H99" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
         <v>109</v>
       </c>
+      <c r="C100" t="s">
+        <v>11</v>
+      </c>
       <c r="G100" t="s">
         <v>10</v>
       </c>
       <c r="H100" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
         <v>110</v>
       </c>
+      <c r="C101" t="s">
+        <v>11</v>
+      </c>
       <c r="G101" t="s">
         <v>10</v>
       </c>
       <c r="H101" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
         <v>111</v>
       </c>
+      <c r="C102" t="s">
+        <v>11</v>
+      </c>
       <c r="G102" t="s">
         <v>10</v>
       </c>
       <c r="H102" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
         <v>112</v>
       </c>
+      <c r="C103" t="s">
+        <v>11</v>
+      </c>
       <c r="G103" t="s">
         <v>10</v>
       </c>
       <c r="H103" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
         <v>113</v>
       </c>
+      <c r="C104" t="s">
+        <v>11</v>
+      </c>
       <c r="G104" t="s">
         <v>10</v>
       </c>
       <c r="H104" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
         <v>114</v>
       </c>
+      <c r="C105" t="s">
+        <v>11</v>
+      </c>
       <c r="G105" t="s">
         <v>10</v>
       </c>
       <c r="H105" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
         <v>115</v>
       </c>
+      <c r="C106" t="s">
+        <v>11</v>
+      </c>
       <c r="G106" t="s">
         <v>10</v>
       </c>
       <c r="H106" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
         <v>116</v>
       </c>
+      <c r="C107" t="s">
+        <v>11</v>
+      </c>
       <c r="G107" t="s">
         <v>10</v>
       </c>
       <c r="H107" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
         <v>117</v>
       </c>
+      <c r="C108" t="s">
+        <v>11</v>
+      </c>
       <c r="G108" t="s">
         <v>10</v>
       </c>
       <c r="H108" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
         <v>118</v>
       </c>
+      <c r="C109" t="s">
+        <v>11</v>
+      </c>
       <c r="G109" t="s">
         <v>10</v>
       </c>
       <c r="H109" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:8">
       <c r="A110" t="s">
         <v>119</v>
       </c>
+      <c r="C110" t="s">
+        <v>11</v>
+      </c>
       <c r="G110" t="s">
         <v>10</v>
       </c>
       <c r="H110" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
         <v>120</v>
       </c>
+      <c r="C111" t="s">
+        <v>11</v>
+      </c>
       <c r="G111" t="s">
         <v>10</v>
       </c>
       <c r="H111" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" spans="1:8">
       <c r="A112" t="s">
         <v>121</v>
       </c>
+      <c r="C112" t="s">
+        <v>11</v>
+      </c>
       <c r="G112" t="s">
         <v>10</v>
       </c>
       <c r="H112" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
         <v>122</v>
       </c>
+      <c r="C113" t="s">
+        <v>11</v>
+      </c>
       <c r="G113" t="s">
         <v>10</v>
       </c>
       <c r="H113" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="114" spans="1:8">
       <c r="A114" t="s">
         <v>123</v>
       </c>
+      <c r="C114" t="s">
+        <v>11</v>
+      </c>
       <c r="G114" t="s">
         <v>10</v>
       </c>
       <c r="H114" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:8">
       <c r="A115" t="s">
         <v>124</v>
       </c>
+      <c r="C115" t="s">
+        <v>11</v>
+      </c>
       <c r="G115" t="s">
         <v>10</v>
       </c>
       <c r="H115" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116" spans="1:8">
       <c r="A116" t="s">
         <v>125</v>
       </c>
+      <c r="C116" t="s">
+        <v>11</v>
+      </c>
       <c r="G116" t="s">
         <v>10</v>
       </c>
       <c r="H116" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117" spans="1:8">
       <c r="A117" t="s">
         <v>126</v>
       </c>
+      <c r="C117" t="s">
+        <v>11</v>
+      </c>
       <c r="G117" t="s">
         <v>10</v>
       </c>
       <c r="H117" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118" spans="1:8">
       <c r="A118" t="s">
         <v>127</v>
       </c>
+      <c r="C118" t="s">
+        <v>11</v>
+      </c>
       <c r="G118" t="s">
         <v>10</v>
       </c>
       <c r="H118" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
         <v>128</v>
       </c>
+      <c r="C119" t="s">
+        <v>11</v>
+      </c>
       <c r="G119" t="s">
         <v>10</v>
       </c>
       <c r="H119" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
         <v>129</v>
       </c>
+      <c r="C120" t="s">
+        <v>11</v>
+      </c>
       <c r="G120" t="s">
         <v>10</v>
       </c>
       <c r="H120" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="121" spans="1:8">
       <c r="A121" t="s">
         <v>130</v>
       </c>
+      <c r="C121" t="s">
+        <v>11</v>
+      </c>
       <c r="G121" t="s">
         <v>10</v>
       </c>
       <c r="H121" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122" spans="1:8">
       <c r="A122" t="s">
         <v>131</v>
       </c>
+      <c r="C122" t="s">
+        <v>11</v>
+      </c>
       <c r="G122" t="s">
         <v>10</v>
       </c>
       <c r="H122" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123" spans="1:8">
       <c r="A123" t="s">
         <v>132</v>
       </c>
+      <c r="C123" t="s">
+        <v>11</v>
+      </c>
       <c r="G123" t="s">
         <v>10</v>
       </c>
       <c r="H123" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="124" spans="1:8">
       <c r="A124" t="s">
         <v>133</v>
       </c>
+      <c r="C124" t="s">
+        <v>11</v>
+      </c>
       <c r="G124" t="s">
         <v>10</v>
       </c>
       <c r="H124" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
         <v>134</v>
       </c>
+      <c r="C125" t="s">
+        <v>11</v>
+      </c>
       <c r="G125" t="s">
         <v>10</v>
       </c>
       <c r="H125" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="A126" t="s">
         <v>135</v>
       </c>
+      <c r="C126" t="s">
+        <v>11</v>
+      </c>
       <c r="G126" t="s">
         <v>10</v>
       </c>
       <c r="H126" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:8">
       <c r="A127" t="s">
         <v>136</v>
       </c>
+      <c r="C127" t="s">
+        <v>11</v>
+      </c>
       <c r="G127" t="s">
         <v>10</v>
       </c>
       <c r="H127" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128" spans="1:8">
       <c r="A128" t="s">
         <v>137</v>
       </c>
+      <c r="C128" t="s">
+        <v>11</v>
+      </c>
       <c r="G128" t="s">
         <v>10</v>
       </c>
       <c r="H128" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="129" spans="1:8">
       <c r="A129" t="s">
         <v>138</v>
       </c>
+      <c r="C129" t="s">
+        <v>11</v>
+      </c>
       <c r="G129" t="s">
         <v>10</v>
       </c>
       <c r="H129" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130" spans="1:8">
       <c r="A130" t="s">
         <v>139</v>
       </c>
+      <c r="C130" t="s">
+        <v>11</v>
+      </c>
       <c r="G130" t="s">
         <v>10</v>
       </c>
       <c r="H130" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" t="s">
         <v>140</v>
       </c>
+      <c r="C131" t="s">
+        <v>11</v>
+      </c>
       <c r="G131" t="s">
         <v>10</v>
       </c>
       <c r="H131" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="132" spans="1:8">
       <c r="A132" t="s">
         <v>141</v>
       </c>
+      <c r="C132" t="s">
+        <v>11</v>
+      </c>
       <c r="G132" t="s">
         <v>10</v>
       </c>
       <c r="H132" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133" spans="1:8">
       <c r="A133" t="s">
         <v>142</v>
       </c>
+      <c r="C133" t="s">
+        <v>11</v>
+      </c>
       <c r="G133" t="s">
         <v>10</v>
       </c>
       <c r="H133" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134" spans="1:8">
       <c r="A134" t="s">
         <v>143</v>
       </c>
+      <c r="C134" t="s">
+        <v>11</v>
+      </c>
       <c r="G134" t="s">
         <v>10</v>
       </c>
       <c r="H134" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="135" spans="1:8">
       <c r="A135" t="s">
         <v>144</v>
       </c>
+      <c r="C135" t="s">
+        <v>11</v>
+      </c>
       <c r="G135" t="s">
         <v>10</v>
       </c>
       <c r="H135" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136" spans="1:8">
       <c r="A136" t="s">
         <v>145</v>
       </c>
+      <c r="C136" t="s">
+        <v>11</v>
+      </c>
       <c r="G136" t="s">
         <v>10</v>
       </c>
       <c r="H136" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="137" spans="1:8">
       <c r="A137" t="s">
         <v>146</v>
       </c>
+      <c r="C137" t="s">
+        <v>11</v>
+      </c>
       <c r="G137" t="s">
         <v>10</v>
       </c>
       <c r="H137" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="138" spans="1:8">
       <c r="A138" t="s">
         <v>147</v>
       </c>
+      <c r="C138" t="s">
+        <v>11</v>
+      </c>
       <c r="G138" t="s">
         <v>10</v>
       </c>
       <c r="H138" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139" spans="1:8">
       <c r="A139" t="s">
         <v>148</v>
       </c>
+      <c r="C139" t="s">
+        <v>11</v>
+      </c>
       <c r="G139" t="s">
         <v>10</v>
       </c>
       <c r="H139" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="140" spans="1:8">
       <c r="A140" t="s">
         <v>149</v>
       </c>
+      <c r="C140" t="s">
+        <v>11</v>
+      </c>
       <c r="G140" t="s">
         <v>10</v>
       </c>
       <c r="H140" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="141" spans="1:8">
       <c r="A141" t="s">
         <v>150</v>
       </c>
+      <c r="C141" t="s">
+        <v>11</v>
+      </c>
       <c r="G141" t="s">
         <v>10</v>
       </c>
       <c r="H141" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="142" spans="1:8">
       <c r="A142" t="s">
         <v>151</v>
       </c>
+      <c r="C142" t="s">
+        <v>11</v>
+      </c>
       <c r="G142" t="s">
         <v>10</v>
       </c>
       <c r="H142" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="143" spans="1:8">
       <c r="A143" t="s">
         <v>152</v>
       </c>
+      <c r="C143" t="s">
+        <v>11</v>
+      </c>
       <c r="G143" t="s">
         <v>10</v>
       </c>
       <c r="H143" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="144" spans="1:8">
       <c r="A144" t="s">
         <v>153</v>
       </c>
+      <c r="C144" t="s">
+        <v>11</v>
+      </c>
       <c r="G144" t="s">
         <v>10</v>
       </c>
       <c r="H144" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:8">
       <c r="A145" t="s">
         <v>154</v>
       </c>
+      <c r="C145" t="s">
+        <v>11</v>
+      </c>
       <c r="G145" t="s">
         <v>10</v>
       </c>
       <c r="H145" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="146" spans="1:8">
       <c r="A146" t="s">
         <v>155</v>
       </c>
+      <c r="C146" t="s">
+        <v>11</v>
+      </c>
       <c r="G146" t="s">
         <v>10</v>
       </c>
       <c r="H146" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="147" spans="1:8">
       <c r="A147" t="s">
         <v>156</v>
       </c>
+      <c r="C147" t="s">
+        <v>11</v>
+      </c>
       <c r="G147" t="s">
         <v>10</v>
       </c>
       <c r="H147" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="148" spans="1:8">
       <c r="A148" t="s">
         <v>157</v>
       </c>
+      <c r="C148" t="s">
+        <v>11</v>
+      </c>
       <c r="G148" t="s">
         <v>10</v>
       </c>
       <c r="H148" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="149" spans="1:8">
       <c r="A149" t="s">
         <v>158</v>
       </c>
+      <c r="C149" t="s">
+        <v>11</v>
+      </c>
       <c r="G149" t="s">
         <v>10</v>
       </c>
       <c r="H149" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:8">
       <c r="A150" t="s">
         <v>159</v>
       </c>
+      <c r="C150" t="s">
+        <v>11</v>
+      </c>
       <c r="G150" t="s">
         <v>10</v>
       </c>
       <c r="H150" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="151" spans="1:8">
       <c r="A151" t="s">
         <v>160</v>
       </c>
+      <c r="C151" t="s">
+        <v>11</v>
+      </c>
       <c r="G151" t="s">
         <v>10</v>
       </c>
       <c r="H151" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152" spans="1:8">
       <c r="A152" t="s">
         <v>161</v>
       </c>
+      <c r="C152" t="s">
+        <v>11</v>
+      </c>
       <c r="G152" t="s">
         <v>10</v>
       </c>
       <c r="H152" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="153" spans="1:8">
       <c r="A153" t="s">
         <v>162</v>
       </c>
+      <c r="C153" t="s">
+        <v>11</v>
+      </c>
       <c r="G153" t="s">
         <v>10</v>
       </c>
       <c r="H153" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="154" spans="1:8">
       <c r="A154" t="s">
         <v>163</v>
       </c>
+      <c r="C154" t="s">
+        <v>11</v>
+      </c>
       <c r="G154" t="s">
         <v>10</v>
       </c>
       <c r="H154" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:8">
       <c r="A155" t="s">
         <v>164</v>
       </c>
+      <c r="C155" t="s">
+        <v>11</v>
+      </c>
       <c r="G155" t="s">
         <v>10</v>
       </c>
       <c r="H155" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="156" spans="1:8">
       <c r="A156" t="s">
         <v>165</v>
       </c>
+      <c r="C156" t="s">
+        <v>11</v>
+      </c>
       <c r="G156" t="s">
         <v>10</v>
       </c>
       <c r="H156" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="157" spans="1:8">
       <c r="A157" t="s">
         <v>166</v>
       </c>
+      <c r="C157" t="s">
+        <v>11</v>
+      </c>
       <c r="G157" t="s">
         <v>10</v>
       </c>
       <c r="H157" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="158" spans="1:8">
       <c r="A158" t="s">
         <v>167</v>
       </c>
+      <c r="C158" t="s">
+        <v>11</v>
+      </c>
       <c r="G158" t="s">
         <v>10</v>
       </c>
       <c r="H158" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="159" spans="1:8">
       <c r="A159" t="s">
         <v>168</v>
       </c>
+      <c r="C159" t="s">
+        <v>11</v>
+      </c>
       <c r="G159" t="s">
         <v>10</v>
       </c>
       <c r="H159" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="160" spans="1:8">
       <c r="A160" t="s">
         <v>169</v>
       </c>
+      <c r="C160" t="s">
+        <v>11</v>
+      </c>
       <c r="G160" t="s">
         <v>10</v>
       </c>
       <c r="H160" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="161" spans="1:8">
       <c r="A161" t="s">
         <v>170</v>
       </c>
+      <c r="C161" t="s">
+        <v>11</v>
+      </c>
       <c r="G161" t="s">
         <v>10</v>
       </c>
       <c r="H161" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="162" spans="1:8">
       <c r="A162" t="s">
         <v>171</v>
       </c>
+      <c r="C162" t="s">
+        <v>11</v>
+      </c>
       <c r="G162" t="s">
         <v>10</v>
       </c>
       <c r="H162" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="163" spans="1:8">
       <c r="A163" t="s">
         <v>172</v>
       </c>
+      <c r="C163" t="s">
+        <v>11</v>
+      </c>
       <c r="G163" t="s">
         <v>10</v>
       </c>
       <c r="H163" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="164" spans="1:8">
       <c r="A164" t="s">
         <v>173</v>
       </c>
+      <c r="C164" t="s">
+        <v>11</v>
+      </c>
       <c r="G164" t="s">
         <v>10</v>
       </c>
       <c r="H164" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="165" spans="1:8">
       <c r="A165" t="s">
         <v>174</v>
       </c>
+      <c r="C165" t="s">
+        <v>11</v>
+      </c>
       <c r="G165" t="s">
         <v>10</v>
       </c>
       <c r="H165" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="166" spans="1:8">
       <c r="A166" t="s">
         <v>175</v>
       </c>
+      <c r="C166" t="s">
+        <v>11</v>
+      </c>
       <c r="G166" t="s">
         <v>10</v>
       </c>
       <c r="H166" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167" spans="1:8">
       <c r="A167" t="s">
         <v>176</v>
       </c>
+      <c r="C167" t="s">
+        <v>11</v>
+      </c>
       <c r="G167" t="s">
         <v>10</v>
       </c>
       <c r="H167" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="168" spans="1:8">
       <c r="A168" t="s">
         <v>177</v>
       </c>
+      <c r="C168" t="s">
+        <v>11</v>
+      </c>
       <c r="G168" t="s">
         <v>10</v>
       </c>
       <c r="H168" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:8">
       <c r="A169" t="s">
         <v>178</v>
       </c>
+      <c r="C169" t="s">
+        <v>11</v>
+      </c>
       <c r="G169" t="s">
         <v>10</v>
       </c>
       <c r="H169" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:8">
       <c r="A170" t="s">
         <v>179</v>
       </c>
+      <c r="C170" t="s">
+        <v>11</v>
+      </c>
       <c r="G170" t="s">
         <v>10</v>
       </c>
       <c r="H170" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:8">
       <c r="A171" t="s">
         <v>180</v>
       </c>
+      <c r="C171" t="s">
+        <v>11</v>
+      </c>
       <c r="G171" t="s">
         <v>10</v>
       </c>
       <c r="H171" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172" spans="1:8">
       <c r="A172" t="s">
         <v>181</v>
       </c>
+      <c r="C172" t="s">
+        <v>11</v>
+      </c>
       <c r="G172" t="s">
         <v>10</v>
       </c>
       <c r="H172" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173" spans="1:8">
       <c r="A173" t="s">
         <v>182</v>
       </c>
+      <c r="C173" t="s">
+        <v>11</v>
+      </c>
       <c r="G173" t="s">
         <v>10</v>
       </c>
       <c r="H173" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="174" spans="1:8">
       <c r="A174" t="s">
         <v>183</v>
       </c>
+      <c r="C174" t="s">
+        <v>11</v>
+      </c>
       <c r="G174" t="s">
         <v>10</v>
       </c>
       <c r="H174" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="175" spans="1:8">
       <c r="A175" t="s">
         <v>184</v>
       </c>
+      <c r="C175" t="s">
+        <v>11</v>
+      </c>
       <c r="G175" t="s">
         <v>10</v>
       </c>
       <c r="H175" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="176" spans="1:8">
       <c r="A176" t="s">
         <v>185</v>
       </c>
+      <c r="C176" t="s">
+        <v>11</v>
+      </c>
       <c r="G176" t="s">
         <v>10</v>
       </c>
       <c r="H176" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="177" spans="1:8">
       <c r="A177" t="s">
         <v>186</v>
       </c>
+      <c r="C177" t="s">
+        <v>11</v>
+      </c>
       <c r="G177" t="s">
         <v>10</v>
       </c>
       <c r="H177" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="178" spans="1:8">
       <c r="A178" t="s">
         <v>187</v>
       </c>
+      <c r="C178" t="s">
+        <v>11</v>
+      </c>
       <c r="G178" t="s">
         <v>10</v>
       </c>
       <c r="H178" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="179" spans="1:8">
       <c r="A179" t="s">
         <v>188</v>
       </c>
+      <c r="C179" t="s">
+        <v>11</v>
+      </c>
       <c r="G179" t="s">
         <v>10</v>
       </c>
       <c r="H179" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180" spans="1:8">
       <c r="A180" t="s">
         <v>189</v>
       </c>
+      <c r="C180" t="s">
+        <v>11</v>
+      </c>
       <c r="G180" t="s">
         <v>10</v>
       </c>
       <c r="H180" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="181" spans="1:8">
       <c r="A181" t="s">
         <v>190</v>
       </c>
+      <c r="C181" t="s">
+        <v>11</v>
+      </c>
       <c r="G181" t="s">
         <v>10</v>
       </c>
       <c r="H181" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="182" spans="1:8">
       <c r="A182" t="s">
         <v>191</v>
       </c>
+      <c r="C182" t="s">
+        <v>11</v>
+      </c>
       <c r="G182" t="s">
         <v>10</v>
       </c>
       <c r="H182" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="183" spans="1:8">
       <c r="A183" t="s">
         <v>192</v>
       </c>
+      <c r="C183" t="s">
+        <v>11</v>
+      </c>
       <c r="G183" t="s">
         <v>10</v>
       </c>
       <c r="H183" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="184" spans="1:8">
       <c r="A184" t="s">
         <v>193</v>
       </c>
+      <c r="C184" t="s">
+        <v>11</v>
+      </c>
       <c r="G184" t="s">
         <v>10</v>
       </c>
       <c r="H184" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="185" spans="1:8">
       <c r="A185" t="s">
         <v>194</v>
       </c>
+      <c r="C185" t="s">
+        <v>11</v>
+      </c>
       <c r="G185" t="s">
         <v>10</v>
       </c>
       <c r="H185" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="186" spans="1:8">
       <c r="A186" t="s">
         <v>195</v>
       </c>
+      <c r="C186" t="s">
+        <v>11</v>
+      </c>
       <c r="G186" t="s">
         <v>10</v>
       </c>
       <c r="H186" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:8">
       <c r="A187" t="s">
         <v>196</v>
       </c>
+      <c r="C187" t="s">
+        <v>11</v>
+      </c>
       <c r="G187" t="s">
         <v>10</v>
       </c>
       <c r="H187" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="188" spans="1:8">
       <c r="A188" t="s">
         <v>197</v>
       </c>
+      <c r="C188" t="s">
+        <v>11</v>
+      </c>
       <c r="G188" t="s">
         <v>10</v>
       </c>
       <c r="H188" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="189" spans="1:8">
       <c r="A189" t="s">
         <v>198</v>
       </c>
+      <c r="C189" t="s">
+        <v>11</v>
+      </c>
       <c r="G189" t="s">
         <v>10</v>
       </c>
       <c r="H189" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="190" spans="1:8">
       <c r="A190" t="s">
         <v>199</v>
       </c>
+      <c r="C190" t="s">
+        <v>11</v>
+      </c>
       <c r="G190" t="s">
         <v>10</v>
       </c>
       <c r="H190" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="191" spans="1:8">
       <c r="A191" t="s">
         <v>200</v>
       </c>
+      <c r="C191" t="s">
+        <v>11</v>
+      </c>
       <c r="G191" t="s">
         <v>10</v>
       </c>
       <c r="H191" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="192" spans="1:8">
       <c r="A192" t="s">
         <v>201</v>
       </c>
+      <c r="C192" t="s">
+        <v>11</v>
+      </c>
       <c r="G192" t="s">
         <v>10</v>
       </c>
       <c r="H192" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193" spans="1:8">
       <c r="A193" t="s">
         <v>202</v>
       </c>
+      <c r="C193" t="s">
+        <v>11</v>
+      </c>
       <c r="G193" t="s">
         <v>10</v>
       </c>
       <c r="H193" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194" spans="1:8">
       <c r="A194" t="s">
         <v>203</v>
       </c>
+      <c r="C194" t="s">
+        <v>11</v>
+      </c>
       <c r="G194" t="s">
         <v>10</v>
       </c>
       <c r="H194" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="195" spans="1:8">
       <c r="A195" t="s">
         <v>204</v>
       </c>
+      <c r="C195" t="s">
+        <v>11</v>
+      </c>
       <c r="G195" t="s">
         <v>10</v>
       </c>
       <c r="H195" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="196" spans="1:8">
       <c r="A196" t="s">
         <v>205</v>
       </c>
+      <c r="C196" t="s">
+        <v>11</v>
+      </c>
       <c r="G196" t="s">
         <v>10</v>
       </c>
       <c r="H196" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="197" spans="1:8">
       <c r="A197" t="s">
         <v>206</v>
       </c>
+      <c r="C197" t="s">
+        <v>11</v>
+      </c>
       <c r="G197" t="s">
         <v>10</v>
       </c>
       <c r="H197" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="198" spans="1:8">
       <c r="A198" t="s">
         <v>207</v>
       </c>
+      <c r="C198" t="s">
+        <v>11</v>
+      </c>
       <c r="G198" t="s">
         <v>10</v>
       </c>
       <c r="H198" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="199" spans="1:8">
       <c r="A199" t="s">
         <v>208</v>
       </c>
+      <c r="C199" t="s">
+        <v>11</v>
+      </c>
       <c r="G199" t="s">
         <v>10</v>
       </c>
       <c r="H199" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="200" spans="1:8">
       <c r="A200" t="s">
         <v>209</v>
       </c>
+      <c r="C200" t="s">
+        <v>11</v>
+      </c>
       <c r="G200" t="s">
         <v>10</v>
       </c>
       <c r="H200" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="201" spans="1:8">
       <c r="A201" t="s">
         <v>210</v>
       </c>
+      <c r="C201" t="s">
+        <v>11</v>
+      </c>
       <c r="G201" t="s">
         <v>10</v>
       </c>
       <c r="H201" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="202" spans="1:8">
       <c r="A202" t="s">
         <v>211</v>
       </c>
+      <c r="C202" t="s">
+        <v>11</v>
+      </c>
       <c r="G202" t="s">
         <v>10</v>
       </c>
       <c r="H202" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203" spans="1:8">
       <c r="A203" t="s">
         <v>212</v>
       </c>
+      <c r="C203" t="s">
+        <v>11</v>
+      </c>
       <c r="G203" t="s">
         <v>10</v>
       </c>
       <c r="H203" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="204" spans="1:8">
       <c r="A204" t="s">
         <v>213</v>
       </c>
+      <c r="C204" t="s">
+        <v>11</v>
+      </c>
       <c r="G204" t="s">
         <v>10</v>
       </c>
       <c r="H204" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="205" spans="1:8">
       <c r="A205" t="s">
         <v>214</v>
       </c>
+      <c r="C205" t="s">
+        <v>11</v>
+      </c>
       <c r="G205" t="s">
         <v>10</v>
       </c>
       <c r="H205" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="206" spans="1:8">
       <c r="A206" t="s">
         <v>215</v>
       </c>
+      <c r="C206" t="s">
+        <v>11</v>
+      </c>
       <c r="G206" t="s">
         <v>10</v>
       </c>
       <c r="H206" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="207" spans="1:8">
       <c r="A207" t="s">
         <v>216</v>
       </c>
+      <c r="C207" t="s">
+        <v>11</v>
+      </c>
       <c r="G207" t="s">
         <v>10</v>
       </c>
       <c r="H207" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="208" spans="1:8">
       <c r="A208" t="s">
         <v>217</v>
       </c>
+      <c r="C208" t="s">
+        <v>11</v>
+      </c>
       <c r="G208" t="s">
         <v>10</v>
       </c>
       <c r="H208" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="209" spans="1:8">
       <c r="A209" t="s">
         <v>218</v>
       </c>
+      <c r="C209" t="s">
+        <v>11</v>
+      </c>
       <c r="G209" t="s">
         <v>10</v>
       </c>
       <c r="H209" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="210" spans="1:8">
       <c r="A210" t="s">
         <v>219</v>
       </c>
+      <c r="C210" t="s">
+        <v>11</v>
+      </c>
       <c r="G210" t="s">
         <v>10</v>
       </c>
       <c r="H210" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="211" spans="1:8">
       <c r="A211" t="s">
         <v>220</v>
       </c>
+      <c r="C211" t="s">
+        <v>11</v>
+      </c>
       <c r="G211" t="s">
         <v>10</v>
       </c>
       <c r="H211" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="212" spans="1:8">
       <c r="A212" t="s">
         <v>221</v>
       </c>
+      <c r="C212" t="s">
+        <v>11</v>
+      </c>
       <c r="G212" t="s">
         <v>10</v>
       </c>
       <c r="H212" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="213" spans="1:8">
       <c r="A213" t="s">
         <v>222</v>
       </c>
+      <c r="C213" t="s">
+        <v>11</v>
+      </c>
       <c r="G213" t="s">
         <v>10</v>
       </c>
       <c r="H213" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="214" spans="1:8">
       <c r="A214" t="s">
         <v>223</v>
       </c>
+      <c r="C214" t="s">
+        <v>11</v>
+      </c>
       <c r="G214" t="s">
         <v>10</v>
       </c>
       <c r="H214" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="215" spans="1:8">
       <c r="A215" t="s">
         <v>224</v>
       </c>
+      <c r="C215" t="s">
+        <v>11</v>
+      </c>
       <c r="G215" t="s">
         <v>10</v>
       </c>
       <c r="H215" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="216" spans="1:8">
       <c r="A216" t="s">
         <v>225</v>
       </c>
+      <c r="C216" t="s">
+        <v>11</v>
+      </c>
       <c r="G216" t="s">
         <v>10</v>
       </c>
       <c r="H216" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="217" spans="1:8">
       <c r="A217" t="s">
         <v>226</v>
       </c>
+      <c r="C217" t="s">
+        <v>11</v>
+      </c>
       <c r="G217" t="s">
         <v>10</v>
       </c>
       <c r="H217" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="218" spans="1:8">
       <c r="A218" t="s">
         <v>227</v>
       </c>
+      <c r="C218" t="s">
+        <v>11</v>
+      </c>
       <c r="G218" t="s">
         <v>10</v>
       </c>
       <c r="H218" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="219" spans="1:8">
       <c r="A219" t="s">
         <v>228</v>
       </c>
+      <c r="C219" t="s">
+        <v>11</v>
+      </c>
       <c r="G219" t="s">
         <v>10</v>
       </c>
       <c r="H219" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="220" spans="1:8">
       <c r="A220" t="s">
         <v>229</v>
       </c>
+      <c r="C220" t="s">
+        <v>11</v>
+      </c>
       <c r="G220" t="s">
         <v>10</v>
       </c>
       <c r="H220" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221" spans="1:8">
       <c r="A221" t="s">
         <v>230</v>
       </c>
+      <c r="C221" t="s">
+        <v>11</v>
+      </c>
       <c r="G221" t="s">
         <v>10</v>
       </c>
       <c r="H221" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:8">
       <c r="A222" t="s">
         <v>231</v>
       </c>
+      <c r="C222" t="s">
+        <v>11</v>
+      </c>
       <c r="G222" t="s">
         <v>10</v>
       </c>
       <c r="H222" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="223" spans="1:8">
       <c r="A223" t="s">
         <v>232</v>
       </c>
+      <c r="C223" t="s">
+        <v>11</v>
+      </c>
       <c r="G223" t="s">
         <v>10</v>
       </c>
       <c r="H223" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="224" spans="1:8">
       <c r="A224" t="s">
         <v>233</v>
       </c>
+      <c r="C224" t="s">
+        <v>11</v>
+      </c>
       <c r="G224" t="s">
         <v>10</v>
       </c>
       <c r="H224" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="225" spans="1:8">
       <c r="A225" t="s">
         <v>234</v>
       </c>
+      <c r="C225" t="s">
+        <v>11</v>
+      </c>
       <c r="G225" t="s">
         <v>10</v>
       </c>
       <c r="H225" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226" spans="1:8">
       <c r="A226" t="s">
         <v>235</v>
       </c>
+      <c r="C226" t="s">
+        <v>11</v>
+      </c>
       <c r="G226" t="s">
         <v>10</v>
       </c>
       <c r="H226" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="227" spans="1:8">
       <c r="A227" t="s">
         <v>236</v>
       </c>
+      <c r="C227" t="s">
+        <v>11</v>
+      </c>
       <c r="G227" t="s">
         <v>10</v>
       </c>
       <c r="H227" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="228" spans="1:8">
       <c r="A228" t="s">
         <v>237</v>
       </c>
+      <c r="C228" t="s">
+        <v>11</v>
+      </c>
       <c r="G228" t="s">
         <v>10</v>
       </c>
       <c r="H228" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="229" spans="1:8">
       <c r="A229" t="s">
         <v>238</v>
       </c>
+      <c r="C229" t="s">
+        <v>11</v>
+      </c>
       <c r="G229" t="s">
         <v>10</v>
       </c>
       <c r="H229" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:8">
       <c r="A230" t="s">
         <v>239</v>
       </c>
+      <c r="C230" t="s">
+        <v>11</v>
+      </c>
       <c r="G230" t="s">
         <v>10</v>
       </c>
       <c r="H230" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:8">
       <c r="A231" t="s">
         <v>240</v>
       </c>
+      <c r="C231" t="s">
+        <v>11</v>
+      </c>
       <c r="G231" t="s">
         <v>10</v>
       </c>
       <c r="H231" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="232" spans="1:8">
       <c r="A232" t="s">
         <v>241</v>
       </c>
+      <c r="C232" t="s">
+        <v>11</v>
+      </c>
       <c r="G232" t="s">
         <v>10</v>
       </c>
       <c r="H232" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="233" spans="1:8">
       <c r="A233" t="s">
         <v>242</v>
       </c>
+      <c r="C233" t="s">
+        <v>11</v>
+      </c>
       <c r="G233" t="s">
         <v>10</v>
       </c>
       <c r="H233" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="234" spans="1:8">
       <c r="A234" t="s">
         <v>243</v>
       </c>
+      <c r="C234" t="s">
+        <v>11</v>
+      </c>
       <c r="G234" t="s">
         <v>10</v>
       </c>
       <c r="H234" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="235" spans="1:8">
       <c r="A235" t="s">
         <v>244</v>
       </c>
+      <c r="C235" t="s">
+        <v>11</v>
+      </c>
       <c r="G235" t="s">
         <v>10</v>
       </c>
       <c r="H235" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="236" spans="1:8">
       <c r="A236" t="s">
         <v>245</v>
       </c>
+      <c r="C236" t="s">
+        <v>11</v>
+      </c>
       <c r="G236" t="s">
         <v>10</v>
       </c>
       <c r="H236" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="237" spans="1:8">
       <c r="A237" t="s">
         <v>246</v>
       </c>
+      <c r="C237" t="s">
+        <v>11</v>
+      </c>
       <c r="G237" t="s">
         <v>10</v>
       </c>
       <c r="H237" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="238" spans="1:8">
       <c r="A238" t="s">
         <v>247</v>
       </c>
+      <c r="C238" t="s">
+        <v>11</v>
+      </c>
       <c r="G238" t="s">
         <v>10</v>
       </c>
       <c r="H238" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="239" spans="1:8">
       <c r="A239" t="s">
         <v>248</v>
       </c>
+      <c r="C239" t="s">
+        <v>11</v>
+      </c>
       <c r="G239" t="s">
         <v>10</v>
       </c>
       <c r="H239" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
         <v>249</v>
       </c>
+      <c r="C240" t="s">
+        <v>11</v>
+      </c>
       <c r="G240" t="s">
         <v>10</v>
       </c>
       <c r="H240" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="241" spans="1:8">
       <c r="A241" t="s">
         <v>250</v>
       </c>
+      <c r="C241" t="s">
+        <v>11</v>
+      </c>
       <c r="G241" t="s">
         <v>10</v>
       </c>
       <c r="H241" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="242" spans="1:8">
       <c r="A242" t="s">
         <v>251</v>
       </c>
+      <c r="C242" t="s">
+        <v>11</v>
+      </c>
       <c r="G242" t="s">
         <v>10</v>
       </c>
       <c r="H242" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="243" spans="1:8">
       <c r="A243" t="s">
         <v>252</v>
       </c>
+      <c r="C243" t="s">
+        <v>11</v>
+      </c>
       <c r="G243" t="s">
         <v>10</v>
       </c>
       <c r="H243" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:8">
       <c r="A244" t="s">
         <v>253</v>
       </c>
+      <c r="C244" t="s">
+        <v>11</v>
+      </c>
       <c r="G244" t="s">
         <v>10</v>
       </c>
       <c r="H244" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="245" spans="1:8">
       <c r="A245" t="s">
         <v>254</v>
       </c>
+      <c r="C245" t="s">
+        <v>11</v>
+      </c>
       <c r="G245" t="s">
         <v>10</v>
       </c>
       <c r="H245" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="246" spans="1:8">
       <c r="A246" t="s">
         <v>255</v>
       </c>
+      <c r="C246" t="s">
+        <v>11</v>
+      </c>
       <c r="G246" t="s">
         <v>10</v>
       </c>
       <c r="H246" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="247" spans="1:8">
       <c r="A247" t="s">
         <v>256</v>
       </c>
+      <c r="C247" t="s">
+        <v>11</v>
+      </c>
       <c r="G247" t="s">
         <v>10</v>
       </c>
       <c r="H247" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="248" spans="1:8">
       <c r="A248" t="s">
         <v>257</v>
       </c>
+      <c r="C248" t="s">
+        <v>11</v>
+      </c>
       <c r="G248" t="s">
         <v>10</v>
       </c>
       <c r="H248" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="249" spans="1:8">
       <c r="A249" t="s">
         <v>258</v>
       </c>
+      <c r="C249" t="s">
+        <v>11</v>
+      </c>
       <c r="G249" t="s">
         <v>10</v>
       </c>
       <c r="H249" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="250" spans="1:8">
       <c r="A250" t="s">
         <v>259</v>
       </c>
+      <c r="C250" t="s">
+        <v>11</v>
+      </c>
       <c r="G250" t="s">
         <v>10</v>
       </c>
       <c r="H250" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="251" spans="1:8">
       <c r="A251" t="s">
         <v>260</v>
       </c>
+      <c r="C251" t="s">
+        <v>11</v>
+      </c>
       <c r="G251" t="s">
         <v>10</v>
       </c>
       <c r="H251" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="252" spans="1:8">
       <c r="A252" t="s">
         <v>261</v>
       </c>
+      <c r="C252" t="s">
+        <v>11</v>
+      </c>
       <c r="G252" t="s">
         <v>10</v>
       </c>
       <c r="H252" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="253" spans="1:8">
       <c r="A253" t="s">
         <v>262</v>
       </c>
+      <c r="C253" t="s">
+        <v>11</v>
+      </c>
       <c r="G253" t="s">
         <v>10</v>
       </c>
       <c r="H253" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="254" spans="1:8">
       <c r="A254" t="s">
         <v>263</v>
       </c>
+      <c r="C254" t="s">
+        <v>11</v>
+      </c>
       <c r="G254" t="s">
         <v>10</v>
       </c>
       <c r="H254" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>